<commit_message>
Filter current counts before intake date
</commit_message>
<xml_diff>
--- a/outputs/tongji_summary/tongji_summary_current.xlsx
+++ b/outputs/tongji_summary/tongji_summary_current.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目标现状对比" sheetId="1" r:id="Ra1867b9b68704924"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据概览" sheetId="2" r:id="R9ac7336f52534751"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="计算规则" sheetId="3" r:id="R10bace7fa5fa413f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目标现状对比" sheetId="1" r:id="R4ab379b55c8543dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据概览" sheetId="2" r:id="R4cff9adabb5445f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="计算规则" sheetId="3" r:id="Rfb3fa1d96a974560"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -931,13 +931,13 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="J12" s="24" t="n">
-        <x:v>727</x:v>
+        <x:v>718</x:v>
       </x:c>
       <x:c r="K12" s="24" t="n">
-        <x:v>627</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="L12" s="28" t="n">
-        <x:v>7.27</x:v>
+        <x:v>7.18</x:v>
       </x:c>
       <x:c r="M12" s="29" t="n">
         <x:v>1</x:v>
@@ -972,13 +972,13 @@
         <x:v>650</x:v>
       </x:c>
       <x:c r="J13" s="24" t="n">
-        <x:v>744</x:v>
+        <x:v>718</x:v>
       </x:c>
       <x:c r="K13" s="24" t="n">
-        <x:v>94</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="L13" s="28" t="n">
-        <x:v>1.1446153846153846</x:v>
+        <x:v>1.1046153846153846</x:v>
       </x:c>
       <x:c r="M13" s="29" t="n">
         <x:v>1</x:v>
@@ -1000,9 +1000,7 @@
       <x:c r="E14" s="12" t="str">
         <x:v>初三</x:v>
       </x:c>
-      <x:c r="F14" s="21" t="str">
-        <x:v>2026-06-21</x:v>
-      </x:c>
+      <x:c r="F14" s="21"/>
       <x:c r="G14" s="21" t="str">
         <x:v>2026-06-30</x:v>
       </x:c>
@@ -1013,13 +1011,13 @@
         <x:v>650</x:v>
       </x:c>
       <x:c r="J14" s="24" t="n">
-        <x:v>82</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K14" s="24" t="n">
-        <x:v>-568</x:v>
+        <x:v>-650</x:v>
       </x:c>
       <x:c r="L14" s="28" t="n">
-        <x:v>0.12615384615384614</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M14" s="29" t="n">
         <x:v>1</x:v>
@@ -1481,13 +1479,13 @@
         <x:v>130</x:v>
       </x:c>
       <x:c r="J26" s="24" t="n">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="K26" s="24" t="n">
-        <x:v>-64</x:v>
+        <x:v>-65</x:v>
       </x:c>
       <x:c r="L26" s="28" t="n">
-        <x:v>0.5076923076923077</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="M26" s="29" t="n">
         <x:v>1</x:v>
@@ -1563,13 +1561,13 @@
         <x:v>130</x:v>
       </x:c>
       <x:c r="J28" s="24" t="n">
-        <x:v>180</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="K28" s="24" t="n">
-        <x:v>50</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="L28" s="28" t="n">
-        <x:v>1.3846153846153846</x:v>
+        <x:v>1.376923076923077</x:v>
       </x:c>
       <x:c r="M28" s="29" t="n">
         <x:v>1</x:v>
@@ -1637,13 +1635,13 @@
         <x:v>800</x:v>
       </x:c>
       <x:c r="J30" s="24" t="n">
-        <x:v>808</x:v>
+        <x:v>668</x:v>
       </x:c>
       <x:c r="K30" s="24" t="n">
-        <x:v>8</x:v>
+        <x:v>-132</x:v>
       </x:c>
       <x:c r="L30" s="28" t="n">
-        <x:v>1.01</x:v>
+        <x:v>0.835</x:v>
       </x:c>
       <x:c r="M30" s="29" t="n">
         <x:v>1</x:v>
@@ -1760,13 +1758,13 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="J33" s="24" t="n">
-        <x:v>479</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="K33" s="24" t="n">
-        <x:v>379</x:v>
+        <x:v>368</x:v>
       </x:c>
       <x:c r="L33" s="28" t="n">
-        <x:v>4.79</x:v>
+        <x:v>4.68</x:v>
       </x:c>
       <x:c r="M33" s="29" t="n">
         <x:v>1</x:v>
@@ -1801,13 +1799,13 @@
         <x:v>700</x:v>
       </x:c>
       <x:c r="J34" s="24" t="n">
-        <x:v>851</x:v>
+        <x:v>836</x:v>
       </x:c>
       <x:c r="K34" s="24" t="n">
-        <x:v>151</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="L34" s="28" t="n">
-        <x:v>1.2157142857142857</x:v>
+        <x:v>1.1942857142857144</x:v>
       </x:c>
       <x:c r="M34" s="29" t="n">
         <x:v>1</x:v>
@@ -1842,13 +1840,13 @@
         <x:v>700</x:v>
       </x:c>
       <x:c r="J35" s="24" t="n">
-        <x:v>515</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="K35" s="24" t="n">
-        <x:v>-185</x:v>
+        <x:v>-198</x:v>
       </x:c>
       <x:c r="L35" s="28" t="n">
-        <x:v>0.7357142857142858</x:v>
+        <x:v>0.7171428571428572</x:v>
       </x:c>
       <x:c r="M35" s="29" t="n">
         <x:v>1</x:v>
@@ -1883,13 +1881,13 @@
         <x:v>220</x:v>
       </x:c>
       <x:c r="J36" s="24" t="n">
-        <x:v>204</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="K36" s="24" t="n">
-        <x:v>-16</x:v>
+        <x:v>-55</x:v>
       </x:c>
       <x:c r="L36" s="28" t="n">
-        <x:v>0.9272727272727272</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M36" s="29" t="n">
         <x:v>1</x:v>
@@ -2121,13 +2119,13 @@
         <x:v>750</x:v>
       </x:c>
       <x:c r="J42" s="24" t="n">
-        <x:v>729</x:v>
+        <x:v>604</x:v>
       </x:c>
       <x:c r="K42" s="24" t="n">
-        <x:v>-21</x:v>
+        <x:v>-146</x:v>
       </x:c>
       <x:c r="L42" s="28" t="n">
-        <x:v>0.972</x:v>
+        <x:v>0.8053333333333333</x:v>
       </x:c>
       <x:c r="M42" s="29" t="n">
         <x:v>1</x:v>
@@ -5939,13 +5937,13 @@
         <x:v>2300</x:v>
       </x:c>
       <x:c r="J156" s="24" t="n">
-        <x:v>2300</x:v>
+        <x:v>1949</x:v>
       </x:c>
       <x:c r="K156" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>-351</x:v>
       </x:c>
       <x:c r="L156" s="28" t="n">
-        <x:v>1</x:v>
+        <x:v>0.8473913043478261</x:v>
       </x:c>
       <x:c r="M156" s="29" t="n">
         <x:v>1</x:v>
@@ -5980,13 +5978,13 @@
         <x:v>2500</x:v>
       </x:c>
       <x:c r="J157" s="24" t="n">
-        <x:v>2503</x:v>
+        <x:v>1981</x:v>
       </x:c>
       <x:c r="K157" s="24" t="n">
-        <x:v>3</x:v>
+        <x:v>-519</x:v>
       </x:c>
       <x:c r="L157" s="28" t="n">
-        <x:v>1.0012</x:v>
+        <x:v>0.7924</x:v>
       </x:c>
       <x:c r="M157" s="29" t="n">
         <x:v>1</x:v>
@@ -6021,13 +6019,13 @@
         <x:v>2000</x:v>
       </x:c>
       <x:c r="J158" s="24" t="n">
-        <x:v>2004</x:v>
+        <x:v>1632</x:v>
       </x:c>
       <x:c r="K158" s="24" t="n">
-        <x:v>4</x:v>
+        <x:v>-368</x:v>
       </x:c>
       <x:c r="L158" s="28" t="n">
-        <x:v>1.002</x:v>
+        <x:v>0.816</x:v>
       </x:c>
       <x:c r="M158" s="29" t="n">
         <x:v>1</x:v>
@@ -6062,13 +6060,13 @@
         <x:v>2300</x:v>
       </x:c>
       <x:c r="J159" s="24" t="n">
-        <x:v>2304</x:v>
+        <x:v>1853</x:v>
       </x:c>
       <x:c r="K159" s="24" t="n">
-        <x:v>4</x:v>
+        <x:v>-447</x:v>
       </x:c>
       <x:c r="L159" s="28" t="n">
-        <x:v>1.0017391304347827</x:v>
+        <x:v>0.8056521739130434</x:v>
       </x:c>
       <x:c r="M159" s="29" t="n">
         <x:v>1</x:v>
@@ -6144,13 +6142,13 @@
         <x:v>150</x:v>
       </x:c>
       <x:c r="J161" s="24" t="n">
-        <x:v>231</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="K161" s="24" t="n">
-        <x:v>81</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="L161" s="28" t="n">
-        <x:v>1.54</x:v>
+        <x:v>1.5333333333333334</x:v>
       </x:c>
       <x:c r="M161" s="29" t="n">
         <x:v>1</x:v>
@@ -6226,13 +6224,13 @@
         <x:v>150</x:v>
       </x:c>
       <x:c r="J163" s="24" t="n">
-        <x:v>166</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="K163" s="24" t="n">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="L163" s="28" t="n">
-        <x:v>1.1066666666666667</x:v>
+        <x:v>1.0666666666666667</x:v>
       </x:c>
       <x:c r="M163" s="29" t="n">
         <x:v>1</x:v>
@@ -6308,13 +6306,13 @@
         <x:v>300</x:v>
       </x:c>
       <x:c r="J165" s="24" t="n">
-        <x:v>249</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="K165" s="24" t="n">
-        <x:v>-51</x:v>
+        <x:v>-56</x:v>
       </x:c>
       <x:c r="L165" s="28" t="n">
-        <x:v>0.83</x:v>
+        <x:v>0.8133333333333334</x:v>
       </x:c>
       <x:c r="M165" s="29" t="n">
         <x:v>1</x:v>
@@ -6390,13 +6388,13 @@
         <x:v>200</x:v>
       </x:c>
       <x:c r="J167" s="24" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K167" s="24" t="n">
-        <x:v>-195</x:v>
+        <x:v>-196</x:v>
       </x:c>
       <x:c r="L167" s="28" t="n">
-        <x:v>0.025</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="M167" s="29" t="n">
         <x:v>1</x:v>
@@ -6618,27 +6616,35 @@
         <x:v>常规外呼</x:v>
       </x:c>
       <x:c r="D173" s="18" t="n">
-        <x:v>18.8</x:v>
+        <x:v>28.8</x:v>
       </x:c>
       <x:c r="E173" s="12" t="str">
-        <x:v>四年级</x:v>
+        <x:v>二年级</x:v>
       </x:c>
       <x:c r="F173" s="21" t="str">
-        <x:v>2026-06-24</x:v>
-      </x:c>
-      <x:c r="G173" s="21"/>
-      <x:c r="H173" s="21"/>
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="G173" s="21" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="H173" s="21" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
       <x:c r="I173" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="J173" s="24" t="n">
-        <x:v>1</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="K173" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L173" s="28"/>
-      <x:c r="M173" s="29"/>
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="L173" s="28" t="n">
+        <x:v>1.225</x:v>
+      </x:c>
+      <x:c r="M173" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="174" ht="15" hidden="0" customHeight="1">
       <x:c r="A174" s="11" t="str">
@@ -6654,7 +6660,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E174" s="12" t="str">
-        <x:v>二年级</x:v>
+        <x:v>三年级</x:v>
       </x:c>
       <x:c r="F174" s="21" t="str">
         <x:v>2026-07-01</x:v>
@@ -6666,16 +6672,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I174" s="24" t="n">
-        <x:v>80</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="J174" s="24" t="n">
-        <x:v>98</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="K174" s="24" t="n">
-        <x:v>18</x:v>
+        <x:v>-52</x:v>
       </x:c>
       <x:c r="L174" s="28" t="n">
-        <x:v>1.225</x:v>
+        <x:v>0.7263157894736842</x:v>
       </x:c>
       <x:c r="M174" s="29" t="n">
         <x:v>1</x:v>
@@ -6695,7 +6701,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E175" s="12" t="str">
-        <x:v>三年级</x:v>
+        <x:v>四年级</x:v>
       </x:c>
       <x:c r="F175" s="21" t="str">
         <x:v>2026-07-01</x:v>
@@ -6707,16 +6713,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I175" s="24" t="n">
-        <x:v>190</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="J175" s="24" t="n">
-        <x:v>138</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="K175" s="24" t="n">
-        <x:v>-52</x:v>
+        <x:v>-4</x:v>
       </x:c>
       <x:c r="L175" s="28" t="n">
-        <x:v>0.7263157894736842</x:v>
+        <x:v>0.9846153846153847</x:v>
       </x:c>
       <x:c r="M175" s="29" t="n">
         <x:v>1</x:v>
@@ -6736,7 +6742,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E176" s="12" t="str">
-        <x:v>四年级</x:v>
+        <x:v>五年级</x:v>
       </x:c>
       <x:c r="F176" s="21" t="str">
         <x:v>2026-07-01</x:v>
@@ -6748,16 +6754,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I176" s="24" t="n">
-        <x:v>260</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="J176" s="24" t="n">
-        <x:v>270</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="K176" s="24" t="n">
-        <x:v>10</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L176" s="28" t="n">
-        <x:v>1.0384615384615385</x:v>
+        <x:v>1.0083333333333333</x:v>
       </x:c>
       <x:c r="M176" s="29" t="n">
         <x:v>1</x:v>
@@ -6777,7 +6783,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E177" s="12" t="str">
-        <x:v>五年级</x:v>
+        <x:v>六年级</x:v>
       </x:c>
       <x:c r="F177" s="21" t="str">
         <x:v>2026-07-01</x:v>
@@ -6789,16 +6795,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I177" s="24" t="n">
-        <x:v>240</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="J177" s="24" t="n">
-        <x:v>242</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="K177" s="24" t="n">
-        <x:v>2</x:v>
+        <x:v>-47</x:v>
       </x:c>
       <x:c r="L177" s="28" t="n">
-        <x:v>1.0083333333333333</x:v>
+        <x:v>0.8192307692307692</x:v>
       </x:c>
       <x:c r="M177" s="29" t="n">
         <x:v>1</x:v>
@@ -6809,40 +6815,40 @@
         <x:v>小学</x:v>
       </x:c>
       <x:c r="B178" s="12" t="str">
-        <x:v>暑_8</x:v>
+        <x:v>暑_9</x:v>
       </x:c>
       <x:c r="C178" s="12" t="str">
-        <x:v>常规外呼</x:v>
+        <x:v>AI托管</x:v>
       </x:c>
       <x:c r="D178" s="18" t="n">
-        <x:v>28.8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E178" s="12" t="str">
-        <x:v>六年级</x:v>
+        <x:v>三年级</x:v>
       </x:c>
       <x:c r="F178" s="21" t="str">
-        <x:v>2026-07-01</x:v>
+        <x:v>2026-07-07</x:v>
       </x:c>
       <x:c r="G178" s="21" t="str">
-        <x:v>2026-07-01</x:v>
+        <x:v>2026-07-08</x:v>
       </x:c>
       <x:c r="H178" s="21" t="str">
-        <x:v>2026-06-25</x:v>
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I178" s="24" t="n">
-        <x:v>260</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="J178" s="24" t="n">
-        <x:v>237</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="K178" s="24" t="n">
-        <x:v>-23</x:v>
+        <x:v>-5</x:v>
       </x:c>
       <x:c r="L178" s="28" t="n">
-        <x:v>0.9115384615384615</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M178" s="29" t="n">
-        <x:v>1</x:v>
+        <x:v>0.8333333333333334</x:v>
       </x:c>
     </x:row>
     <x:row r="179" ht="15" hidden="0" customHeight="1">
@@ -6859,7 +6865,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E179" s="12" t="str">
-        <x:v>三年级</x:v>
+        <x:v>四年级</x:v>
       </x:c>
       <x:c r="F179" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -6871,16 +6877,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I179" s="24" t="n">
-        <x:v>20</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="J179" s="24" t="n">
-        <x:v>15</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="K179" s="24" t="n">
-        <x:v>-5</x:v>
+        <x:v>-56</x:v>
       </x:c>
       <x:c r="L179" s="28" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.4909090909090909</x:v>
       </x:c>
       <x:c r="M179" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -6900,7 +6906,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E180" s="12" t="str">
-        <x:v>四年级</x:v>
+        <x:v>五年级</x:v>
       </x:c>
       <x:c r="F180" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -6941,7 +6947,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E181" s="12" t="str">
-        <x:v>五年级</x:v>
+        <x:v>六年级</x:v>
       </x:c>
       <x:c r="F181" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -6956,13 +6962,13 @@
         <x:v>110</x:v>
       </x:c>
       <x:c r="J181" s="24" t="n">
-        <x:v>54</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="K181" s="24" t="n">
-        <x:v>-56</x:v>
+        <x:v>-47</x:v>
       </x:c>
       <x:c r="L181" s="28" t="n">
-        <x:v>0.4909090909090909</x:v>
+        <x:v>0.5727272727272728</x:v>
       </x:c>
       <x:c r="M181" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -6976,13 +6982,13 @@
         <x:v>暑_9</x:v>
       </x:c>
       <x:c r="C182" s="12" t="str">
-        <x:v>AI托管</x:v>
+        <x:v>LEC内测</x:v>
       </x:c>
       <x:c r="D182" s="18" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E182" s="12" t="str">
-        <x:v>六年级</x:v>
+        <x:v>三年级</x:v>
       </x:c>
       <x:c r="F182" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -6994,16 +7000,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I182" s="24" t="n">
-        <x:v>110</x:v>
+        <x:v>2520</x:v>
       </x:c>
       <x:c r="J182" s="24" t="n">
-        <x:v>63</x:v>
+        <x:v>2510</x:v>
       </x:c>
       <x:c r="K182" s="24" t="n">
-        <x:v>-47</x:v>
+        <x:v>-10</x:v>
       </x:c>
       <x:c r="L182" s="28" t="n">
-        <x:v>0.5727272727272728</x:v>
+        <x:v>0.996031746031746</x:v>
       </x:c>
       <x:c r="M182" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -7023,7 +7029,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E183" s="12" t="str">
-        <x:v>三年级</x:v>
+        <x:v>四年级</x:v>
       </x:c>
       <x:c r="F183" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -7035,16 +7041,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I183" s="24" t="n">
-        <x:v>2520</x:v>
+        <x:v>2720</x:v>
       </x:c>
       <x:c r="J183" s="24" t="n">
-        <x:v>2510</x:v>
+        <x:v>2713</x:v>
       </x:c>
       <x:c r="K183" s="24" t="n">
-        <x:v>-10</x:v>
+        <x:v>-7</x:v>
       </x:c>
       <x:c r="L183" s="28" t="n">
-        <x:v>0.996031746031746</x:v>
+        <x:v>0.9974264705882353</x:v>
       </x:c>
       <x:c r="M183" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -7064,7 +7070,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E184" s="12" t="str">
-        <x:v>四年级</x:v>
+        <x:v>五年级</x:v>
       </x:c>
       <x:c r="F184" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -7076,16 +7082,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I184" s="24" t="n">
-        <x:v>2720</x:v>
+        <x:v>2530</x:v>
       </x:c>
       <x:c r="J184" s="24" t="n">
-        <x:v>2713</x:v>
+        <x:v>2312</x:v>
       </x:c>
       <x:c r="K184" s="24" t="n">
-        <x:v>-7</x:v>
+        <x:v>-218</x:v>
       </x:c>
       <x:c r="L184" s="28" t="n">
-        <x:v>0.9974264705882353</x:v>
+        <x:v>0.9138339920948617</x:v>
       </x:c>
       <x:c r="M184" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -7105,7 +7111,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E185" s="12" t="str">
-        <x:v>五年级</x:v>
+        <x:v>六年级</x:v>
       </x:c>
       <x:c r="F185" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -7117,16 +7123,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I185" s="24" t="n">
-        <x:v>2530</x:v>
+        <x:v>2050</x:v>
       </x:c>
       <x:c r="J185" s="24" t="n">
-        <x:v>2312</x:v>
+        <x:v>2031</x:v>
       </x:c>
       <x:c r="K185" s="24" t="n">
-        <x:v>-218</x:v>
+        <x:v>-19</x:v>
       </x:c>
       <x:c r="L185" s="28" t="n">
-        <x:v>0.9138339920948617</x:v>
+        <x:v>0.9907317073170732</x:v>
       </x:c>
       <x:c r="M185" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -7140,38 +7146,30 @@
         <x:v>暑_9</x:v>
       </x:c>
       <x:c r="C186" s="12" t="str">
-        <x:v>LEC内测</x:v>
+        <x:v>LLM外呼</x:v>
       </x:c>
       <x:c r="D186" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>9.9</x:v>
       </x:c>
       <x:c r="E186" s="12" t="str">
-        <x:v>六年级</x:v>
+        <x:v>二年级</x:v>
       </x:c>
       <x:c r="F186" s="21" t="str">
-        <x:v>2026-07-07</x:v>
-      </x:c>
-      <x:c r="G186" s="21" t="str">
-        <x:v>2026-07-08</x:v>
-      </x:c>
-      <x:c r="H186" s="21" t="str">
-        <x:v>2026-07-02</x:v>
-      </x:c>
+        <x:v>2026-07-03</x:v>
+      </x:c>
+      <x:c r="G186" s="21"/>
+      <x:c r="H186" s="21"/>
       <x:c r="I186" s="24" t="n">
-        <x:v>2050</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J186" s="24" t="n">
-        <x:v>2031</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="K186" s="24" t="n">
-        <x:v>-19</x:v>
-      </x:c>
-      <x:c r="L186" s="28" t="n">
-        <x:v>0.9907317073170732</x:v>
-      </x:c>
-      <x:c r="M186" s="29" t="n">
-        <x:v>0.8333333333333334</x:v>
-      </x:c>
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="L186" s="28"/>
+      <x:c r="M186" s="29"/>
     </x:row>
     <x:row r="187" ht="15" hidden="0" customHeight="1">
       <x:c r="A187" s="11" t="str">
@@ -7187,24 +7185,32 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E187" s="12" t="str">
-        <x:v>二年级</x:v>
+        <x:v>三年级</x:v>
       </x:c>
       <x:c r="F187" s="21" t="str">
-        <x:v>2026-07-03</x:v>
-      </x:c>
-      <x:c r="G187" s="21"/>
-      <x:c r="H187" s="21"/>
+        <x:v>2026-07-07</x:v>
+      </x:c>
+      <x:c r="G187" s="21" t="str">
+        <x:v>2026-07-08</x:v>
+      </x:c>
+      <x:c r="H187" s="21" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
       <x:c r="I187" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="J187" s="24" t="n">
-        <x:v>67</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="K187" s="24" t="n">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="L187" s="28"/>
-      <x:c r="M187" s="29"/>
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="L187" s="28" t="n">
+        <x:v>1.4133333333333333</x:v>
+      </x:c>
+      <x:c r="M187" s="29" t="n">
+        <x:v>0.8333333333333334</x:v>
+      </x:c>
     </x:row>
     <x:row r="188" ht="15" hidden="0" customHeight="1">
       <x:c r="A188" s="11" t="str">
@@ -7220,7 +7226,7 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E188" s="12" t="str">
-        <x:v>三年级</x:v>
+        <x:v>四年级</x:v>
       </x:c>
       <x:c r="F188" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -7232,16 +7238,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I188" s="24" t="n">
-        <x:v>150</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="J188" s="24" t="n">
-        <x:v>213</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="K188" s="24" t="n">
-        <x:v>63</x:v>
+        <x:v>-115</x:v>
       </x:c>
       <x:c r="L188" s="28" t="n">
-        <x:v>1.42</x:v>
+        <x:v>0.6714285714285714</x:v>
       </x:c>
       <x:c r="M188" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -7261,7 +7267,7 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E189" s="12" t="str">
-        <x:v>四年级</x:v>
+        <x:v>五年级</x:v>
       </x:c>
       <x:c r="F189" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -7273,16 +7279,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I189" s="24" t="n">
-        <x:v>350</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="J189" s="24" t="n">
-        <x:v>243</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="K189" s="24" t="n">
-        <x:v>-107</x:v>
+        <x:v>-57</x:v>
       </x:c>
       <x:c r="L189" s="28" t="n">
-        <x:v>0.6942857142857143</x:v>
+        <x:v>0.772</x:v>
       </x:c>
       <x:c r="M189" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -7302,10 +7308,10 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E190" s="12" t="str">
-        <x:v>五年级</x:v>
+        <x:v>六年级</x:v>
       </x:c>
       <x:c r="F190" s="21" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-07-06</x:v>
       </x:c>
       <x:c r="G190" s="21" t="str">
         <x:v>2026-07-08</x:v>
@@ -7317,13 +7323,13 @@
         <x:v>250</x:v>
       </x:c>
       <x:c r="J190" s="24" t="n">
-        <x:v>204</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="K190" s="24" t="n">
-        <x:v>-46</x:v>
+        <x:v>-183</x:v>
       </x:c>
       <x:c r="L190" s="28" t="n">
-        <x:v>0.816</x:v>
+        <x:v>0.268</x:v>
       </x:c>
       <x:c r="M190" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -7337,38 +7343,30 @@
         <x:v>暑_9</x:v>
       </x:c>
       <x:c r="C191" s="12" t="str">
-        <x:v>LLM外呼</x:v>
+        <x:v>常规外呼</x:v>
       </x:c>
       <x:c r="D191" s="18" t="n">
-        <x:v>9.9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E191" s="12" t="str">
-        <x:v>六年级</x:v>
+        <x:v>三年级</x:v>
       </x:c>
       <x:c r="F191" s="21" t="str">
-        <x:v>2026-07-06</x:v>
-      </x:c>
-      <x:c r="G191" s="21" t="str">
-        <x:v>2026-07-08</x:v>
-      </x:c>
-      <x:c r="H191" s="21" t="str">
-        <x:v>2026-07-02</x:v>
-      </x:c>
+        <x:v>2026-07-05</x:v>
+      </x:c>
+      <x:c r="G191" s="21"/>
+      <x:c r="H191" s="21"/>
       <x:c r="I191" s="24" t="n">
-        <x:v>250</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J191" s="24" t="n">
-        <x:v>230</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="K191" s="24" t="n">
-        <x:v>-20</x:v>
-      </x:c>
-      <x:c r="L191" s="28" t="n">
-        <x:v>0.92</x:v>
-      </x:c>
-      <x:c r="M191" s="29" t="n">
-        <x:v>0.8333333333333334</x:v>
-      </x:c>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="L191" s="28"/>
+      <x:c r="M191" s="29"/>
     </x:row>
     <x:row r="192" ht="15" hidden="0" customHeight="1">
       <x:c r="A192" s="11" t="str">
@@ -7384,10 +7382,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E192" s="12" t="str">
-        <x:v>三年级</x:v>
+        <x:v>四年级</x:v>
       </x:c>
       <x:c r="F192" s="21" t="str">
-        <x:v>2026-07-05</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
       <x:c r="G192" s="21"/>
       <x:c r="H192" s="21"/>
@@ -7395,10 +7393,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J192" s="24" t="n">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="K192" s="24" t="n">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="L192" s="28"/>
       <x:c r="M192" s="29"/>
@@ -7417,10 +7415,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E193" s="12" t="str">
-        <x:v>四年级</x:v>
+        <x:v>五年级</x:v>
       </x:c>
       <x:c r="F193" s="21" t="str">
-        <x:v>2026-07-04</x:v>
+        <x:v>2026-07-07</x:v>
       </x:c>
       <x:c r="G193" s="21"/>
       <x:c r="H193" s="21"/>
@@ -7428,10 +7426,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J193" s="24" t="n">
-        <x:v>7</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="K193" s="24" t="n">
-        <x:v>7</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="L193" s="28"/>
       <x:c r="M193" s="29"/>
@@ -7450,10 +7448,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E194" s="12" t="str">
-        <x:v>五年级</x:v>
+        <x:v>六年级</x:v>
       </x:c>
       <x:c r="F194" s="21" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-07-05</x:v>
       </x:c>
       <x:c r="G194" s="21"/>
       <x:c r="H194" s="21"/>
@@ -7461,10 +7459,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J194" s="24" t="n">
-        <x:v>12</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="K194" s="24" t="n">
-        <x:v>12</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="L194" s="28"/>
       <x:c r="M194" s="29"/>
@@ -7480,27 +7478,35 @@
         <x:v>常规外呼</x:v>
       </x:c>
       <x:c r="D195" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>28.8</x:v>
       </x:c>
       <x:c r="E195" s="12" t="str">
-        <x:v>六年级</x:v>
+        <x:v>二年级</x:v>
       </x:c>
       <x:c r="F195" s="21" t="str">
-        <x:v>2026-07-05</x:v>
-      </x:c>
-      <x:c r="G195" s="21"/>
-      <x:c r="H195" s="21"/>
+        <x:v>2026-07-07</x:v>
+      </x:c>
+      <x:c r="G195" s="21" t="str">
+        <x:v>2026-07-08</x:v>
+      </x:c>
+      <x:c r="H195" s="21" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
       <x:c r="I195" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="J195" s="24" t="n">
-        <x:v>19</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="K195" s="24" t="n">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="L195" s="28"/>
-      <x:c r="M195" s="29"/>
+        <x:v>-4</x:v>
+      </x:c>
+      <x:c r="L195" s="28" t="n">
+        <x:v>0.96</x:v>
+      </x:c>
+      <x:c r="M195" s="29" t="n">
+        <x:v>0.8333333333333334</x:v>
+      </x:c>
     </x:row>
     <x:row r="196" ht="15" hidden="0" customHeight="1">
       <x:c r="A196" s="11" t="str">
@@ -7516,7 +7522,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E196" s="12" t="str">
-        <x:v>二年级</x:v>
+        <x:v>三年级</x:v>
       </x:c>
       <x:c r="F196" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -7528,16 +7534,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I196" s="24" t="n">
-        <x:v>100</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="J196" s="24" t="n">
-        <x:v>96</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="K196" s="24" t="n">
-        <x:v>-4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L196" s="28" t="n">
-        <x:v>0.96</x:v>
+        <x:v>1.0217391304347827</x:v>
       </x:c>
       <x:c r="M196" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -7557,7 +7563,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E197" s="12" t="str">
-        <x:v>三年级</x:v>
+        <x:v>四年级</x:v>
       </x:c>
       <x:c r="F197" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -7569,16 +7575,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I197" s="24" t="n">
-        <x:v>230</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="J197" s="24" t="n">
-        <x:v>235</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="K197" s="24" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L197" s="28" t="n">
-        <x:v>1.0217391304347827</x:v>
+        <x:v>1.009090909090909</x:v>
       </x:c>
       <x:c r="M197" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -7598,7 +7604,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E198" s="12" t="str">
-        <x:v>四年级</x:v>
+        <x:v>五年级</x:v>
       </x:c>
       <x:c r="F198" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -7613,13 +7619,13 @@
         <x:v>330</x:v>
       </x:c>
       <x:c r="J198" s="24" t="n">
-        <x:v>333</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="K198" s="24" t="n">
-        <x:v>3</x:v>
+        <x:v>-9</x:v>
       </x:c>
       <x:c r="L198" s="28" t="n">
-        <x:v>1.009090909090909</x:v>
+        <x:v>0.9727272727272728</x:v>
       </x:c>
       <x:c r="M198" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -7639,7 +7645,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E199" s="12" t="str">
-        <x:v>五年级</x:v>
+        <x:v>六年级</x:v>
       </x:c>
       <x:c r="F199" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -7651,16 +7657,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I199" s="24" t="n">
-        <x:v>330</x:v>
+        <x:v>420</x:v>
       </x:c>
       <x:c r="J199" s="24" t="n">
-        <x:v>321</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="K199" s="24" t="n">
-        <x:v>-9</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="L199" s="28" t="n">
-        <x:v>0.9727272727272728</x:v>
+        <x:v>1.0642857142857143</x:v>
       </x:c>
       <x:c r="M199" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -7668,44 +7674,36 @@
     </x:row>
     <x:row r="200" ht="15" hidden="0" customHeight="1">
       <x:c r="A200" s="11" t="str">
-        <x:v>小学</x:v>
+        <x:v>自拼</x:v>
       </x:c>
       <x:c r="B200" s="12" t="str">
-        <x:v>暑_9</x:v>
+        <x:v>暑_10</x:v>
       </x:c>
       <x:c r="C200" s="12" t="str">
         <x:v>常规外呼</x:v>
       </x:c>
       <x:c r="D200" s="18" t="n">
-        <x:v>28.8</x:v>
+        <x:v>29.9</x:v>
       </x:c>
       <x:c r="E200" s="12" t="str">
-        <x:v>六年级</x:v>
+        <x:v>一年级</x:v>
       </x:c>
       <x:c r="F200" s="21" t="str">
         <x:v>2026-07-07</x:v>
       </x:c>
-      <x:c r="G200" s="21" t="str">
-        <x:v>2026-07-08</x:v>
-      </x:c>
-      <x:c r="H200" s="21" t="str">
-        <x:v>2026-07-02</x:v>
-      </x:c>
+      <x:c r="G200" s="21"/>
+      <x:c r="H200" s="21"/>
       <x:c r="I200" s="24" t="n">
-        <x:v>420</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J200" s="24" t="n">
-        <x:v>447</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K200" s="24" t="n">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="L200" s="28" t="n">
-        <x:v>1.0642857142857143</x:v>
-      </x:c>
-      <x:c r="M200" s="29" t="n">
-        <x:v>0.8333333333333334</x:v>
-      </x:c>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L200" s="28"/>
+      <x:c r="M200" s="29"/>
     </x:row>
     <x:row r="201" ht="15" hidden="0" customHeight="1">
       <x:c r="A201" s="11" t="str">
@@ -7721,7 +7719,7 @@
         <x:v>29.9</x:v>
       </x:c>
       <x:c r="E201" s="12" t="str">
-        <x:v>一年级</x:v>
+        <x:v>三年级</x:v>
       </x:c>
       <x:c r="F201" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -7732,10 +7730,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J201" s="24" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K201" s="24" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L201" s="28"/>
       <x:c r="M201" s="29"/>
@@ -7754,7 +7752,7 @@
         <x:v>29.9</x:v>
       </x:c>
       <x:c r="E202" s="12" t="str">
-        <x:v>三年级</x:v>
+        <x:v>四年级</x:v>
       </x:c>
       <x:c r="F202" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -7765,10 +7763,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J202" s="24" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K202" s="24" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L202" s="28"/>
       <x:c r="M202" s="29"/>
@@ -7778,19 +7776,19 @@
         <x:v>自拼</x:v>
       </x:c>
       <x:c r="B203" s="12" t="str">
-        <x:v>暑_10</x:v>
+        <x:v>暑_7</x:v>
       </x:c>
       <x:c r="C203" s="12" t="str">
-        <x:v>常规外呼</x:v>
+        <x:v>LEC内测</x:v>
       </x:c>
       <x:c r="D203" s="18" t="n">
-        <x:v>29.9</x:v>
+        <x:v>9.9</x:v>
       </x:c>
       <x:c r="E203" s="12" t="str">
-        <x:v>四年级</x:v>
+        <x:v>一年级</x:v>
       </x:c>
       <x:c r="F203" s="21" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
       <x:c r="G203" s="21"/>
       <x:c r="H203" s="21"/>
@@ -7798,10 +7796,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J203" s="24" t="n">
-        <x:v>1</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="K203" s="24" t="n">
-        <x:v>1</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="L203" s="28"/>
       <x:c r="M203" s="29"/>
@@ -7820,10 +7818,10 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E204" s="12" t="str">
-        <x:v>一年级</x:v>
+        <x:v>三年级</x:v>
       </x:c>
       <x:c r="F204" s="21" t="str">
-        <x:v>2026-06-22</x:v>
+        <x:v>2026-06-23</x:v>
       </x:c>
       <x:c r="G204" s="21"/>
       <x:c r="H204" s="21"/>
@@ -7831,10 +7829,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J204" s="24" t="n">
-        <x:v>218</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="K204" s="24" t="n">
-        <x:v>218</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="L204" s="28"/>
       <x:c r="M204" s="29"/>
@@ -7853,7 +7851,7 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E205" s="12" t="str">
-        <x:v>三年级</x:v>
+        <x:v>四年级</x:v>
       </x:c>
       <x:c r="F205" s="21" t="str">
         <x:v>2026-06-23</x:v>
@@ -7864,10 +7862,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J205" s="24" t="n">
-        <x:v>79</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="K205" s="24" t="n">
-        <x:v>79</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L205" s="28"/>
       <x:c r="M205" s="29"/>
@@ -7880,16 +7878,16 @@
         <x:v>暑_7</x:v>
       </x:c>
       <x:c r="C206" s="12" t="str">
-        <x:v>LEC内测</x:v>
+        <x:v>WB</x:v>
       </x:c>
       <x:c r="D206" s="18" t="n">
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E206" s="12" t="str">
-        <x:v>四年级</x:v>
+        <x:v>一年级</x:v>
       </x:c>
       <x:c r="F206" s="21" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
       <x:c r="G206" s="21"/>
       <x:c r="H206" s="21"/>
@@ -7897,10 +7895,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J206" s="24" t="n">
-        <x:v>32</x:v>
+        <x:v>314</x:v>
       </x:c>
       <x:c r="K206" s="24" t="n">
-        <x:v>32</x:v>
+        <x:v>314</x:v>
       </x:c>
       <x:c r="L206" s="28"/>
       <x:c r="M206" s="29"/>
@@ -7919,10 +7917,10 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E207" s="12" t="str">
-        <x:v>一年级</x:v>
+        <x:v>三年级</x:v>
       </x:c>
       <x:c r="F207" s="21" t="str">
-        <x:v>2026-06-22</x:v>
+        <x:v>2026-06-23</x:v>
       </x:c>
       <x:c r="G207" s="21"/>
       <x:c r="H207" s="21"/>
@@ -7930,10 +7928,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J207" s="24" t="n">
-        <x:v>314</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="K207" s="24" t="n">
-        <x:v>314</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="L207" s="28"/>
       <x:c r="M207" s="29"/>
@@ -7952,7 +7950,7 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E208" s="12" t="str">
-        <x:v>三年级</x:v>
+        <x:v>四年级</x:v>
       </x:c>
       <x:c r="F208" s="21" t="str">
         <x:v>2026-06-23</x:v>
@@ -7963,10 +7961,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J208" s="24" t="n">
-        <x:v>116</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="K208" s="24" t="n">
-        <x:v>116</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="L208" s="28"/>
       <x:c r="M208" s="29"/>
@@ -7979,16 +7977,16 @@
         <x:v>暑_7</x:v>
       </x:c>
       <x:c r="C209" s="12" t="str">
-        <x:v>WB</x:v>
+        <x:v>外部微转-*</x:v>
       </x:c>
       <x:c r="D209" s="18" t="n">
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E209" s="12" t="str">
-        <x:v>四年级</x:v>
+        <x:v>一年级</x:v>
       </x:c>
       <x:c r="F209" s="21" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-06-21</x:v>
       </x:c>
       <x:c r="G209" s="21"/>
       <x:c r="H209" s="21"/>
@@ -7996,10 +7994,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J209" s="24" t="n">
-        <x:v>89</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="K209" s="24" t="n">
-        <x:v>89</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L209" s="28"/>
       <x:c r="M209" s="29"/>
@@ -8018,10 +8016,10 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E210" s="12" t="str">
-        <x:v>一年级</x:v>
+        <x:v>三年级</x:v>
       </x:c>
       <x:c r="F210" s="21" t="str">
-        <x:v>2026-06-21</x:v>
+        <x:v>2026-06-23</x:v>
       </x:c>
       <x:c r="G210" s="21"/>
       <x:c r="H210" s="21"/>
@@ -8029,10 +8027,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J210" s="24" t="n">
-        <x:v>32</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="K210" s="24" t="n">
-        <x:v>32</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="L210" s="28"/>
       <x:c r="M210" s="29"/>
@@ -8051,7 +8049,7 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E211" s="12" t="str">
-        <x:v>三年级</x:v>
+        <x:v>四年级</x:v>
       </x:c>
       <x:c r="F211" s="21" t="str">
         <x:v>2026-06-23</x:v>
@@ -8062,10 +8060,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J211" s="24" t="n">
-        <x:v>8</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="K211" s="24" t="n">
-        <x:v>8</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="L211" s="28"/>
       <x:c r="M211" s="29"/>
@@ -8078,16 +8076,16 @@
         <x:v>暑_7</x:v>
       </x:c>
       <x:c r="C212" s="12" t="str">
-        <x:v>外部微转-*</x:v>
+        <x:v>常规外呼</x:v>
       </x:c>
       <x:c r="D212" s="18" t="n">
-        <x:v>9.9</x:v>
+        <x:v>29.9</x:v>
       </x:c>
       <x:c r="E212" s="12" t="str">
-        <x:v>四年级</x:v>
+        <x:v>一年级</x:v>
       </x:c>
       <x:c r="F212" s="21" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-06-21</x:v>
       </x:c>
       <x:c r="G212" s="21"/>
       <x:c r="H212" s="21"/>
@@ -8095,10 +8093,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J212" s="24" t="n">
-        <x:v>11</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="K212" s="24" t="n">
-        <x:v>11</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="L212" s="28"/>
       <x:c r="M212" s="29"/>
@@ -8117,10 +8115,10 @@
         <x:v>29.9</x:v>
       </x:c>
       <x:c r="E213" s="12" t="str">
-        <x:v>一年级</x:v>
+        <x:v>三年级</x:v>
       </x:c>
       <x:c r="F213" s="21" t="str">
-        <x:v>2026-06-21</x:v>
+        <x:v>2026-06-20</x:v>
       </x:c>
       <x:c r="G213" s="21"/>
       <x:c r="H213" s="21"/>
@@ -8128,10 +8126,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J213" s="24" t="n">
-        <x:v>7</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K213" s="24" t="n">
-        <x:v>7</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L213" s="28"/>
       <x:c r="M213" s="29"/>
@@ -8150,10 +8148,10 @@
         <x:v>29.9</x:v>
       </x:c>
       <x:c r="E214" s="12" t="str">
-        <x:v>三年级</x:v>
+        <x:v>四年级</x:v>
       </x:c>
       <x:c r="F214" s="21" t="str">
-        <x:v>2026-06-20</x:v>
+        <x:v>2026-06-23</x:v>
       </x:c>
       <x:c r="G214" s="21"/>
       <x:c r="H214" s="21"/>
@@ -8161,10 +8159,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J214" s="24" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K214" s="24" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L214" s="28"/>
       <x:c r="M214" s="29"/>
@@ -8174,19 +8172,19 @@
         <x:v>自拼</x:v>
       </x:c>
       <x:c r="B215" s="12" t="str">
-        <x:v>暑_7</x:v>
+        <x:v>暑_8</x:v>
       </x:c>
       <x:c r="C215" s="12" t="str">
-        <x:v>常规外呼</x:v>
+        <x:v>WB</x:v>
       </x:c>
       <x:c r="D215" s="18" t="n">
-        <x:v>29.9</x:v>
+        <x:v>9.9</x:v>
       </x:c>
       <x:c r="E215" s="12" t="str">
-        <x:v>四年级</x:v>
+        <x:v>一年级</x:v>
       </x:c>
       <x:c r="F215" s="21" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-06-30</x:v>
       </x:c>
       <x:c r="G215" s="21"/>
       <x:c r="H215" s="21"/>
@@ -8194,10 +8192,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J215" s="24" t="n">
-        <x:v>3</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="K215" s="24" t="n">
-        <x:v>3</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="L215" s="28"/>
       <x:c r="M215" s="29"/>
@@ -8216,7 +8214,7 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E216" s="12" t="str">
-        <x:v>一年级</x:v>
+        <x:v>三年级</x:v>
       </x:c>
       <x:c r="F216" s="21" t="str">
         <x:v>2026-06-30</x:v>
@@ -8227,10 +8225,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J216" s="24" t="n">
-        <x:v>295</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="K216" s="24" t="n">
-        <x:v>295</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="L216" s="28"/>
       <x:c r="M216" s="29"/>
@@ -8249,7 +8247,7 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E217" s="12" t="str">
-        <x:v>三年级</x:v>
+        <x:v>四年级</x:v>
       </x:c>
       <x:c r="F217" s="21" t="str">
         <x:v>2026-06-30</x:v>
@@ -8260,10 +8258,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J217" s="24" t="n">
-        <x:v>47</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="K217" s="24" t="n">
-        <x:v>47</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="L217" s="28"/>
       <x:c r="M217" s="29"/>
@@ -8276,13 +8274,13 @@
         <x:v>暑_8</x:v>
       </x:c>
       <x:c r="C218" s="12" t="str">
-        <x:v>WB</x:v>
+        <x:v>常规外呼</x:v>
       </x:c>
       <x:c r="D218" s="18" t="n">
-        <x:v>9.9</x:v>
+        <x:v>29.9</x:v>
       </x:c>
       <x:c r="E218" s="12" t="str">
-        <x:v>四年级</x:v>
+        <x:v>一年级</x:v>
       </x:c>
       <x:c r="F218" s="21" t="str">
         <x:v>2026-06-30</x:v>
@@ -8293,10 +8291,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J218" s="24" t="n">
-        <x:v>50</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="K218" s="24" t="n">
-        <x:v>50</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="L218" s="28"/>
       <x:c r="M218" s="29"/>
@@ -8315,7 +8313,7 @@
         <x:v>29.9</x:v>
       </x:c>
       <x:c r="E219" s="12" t="str">
-        <x:v>一年级</x:v>
+        <x:v>三年级</x:v>
       </x:c>
       <x:c r="F219" s="21" t="str">
         <x:v>2026-06-30</x:v>
@@ -8326,10 +8324,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J219" s="24" t="n">
-        <x:v>13</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="K219" s="24" t="n">
-        <x:v>13</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="L219" s="28"/>
       <x:c r="M219" s="29"/>
@@ -8348,7 +8346,7 @@
         <x:v>29.9</x:v>
       </x:c>
       <x:c r="E220" s="12" t="str">
-        <x:v>三年级</x:v>
+        <x:v>四年级</x:v>
       </x:c>
       <x:c r="F220" s="21" t="str">
         <x:v>2026-06-30</x:v>
@@ -8359,10 +8357,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J220" s="24" t="n">
-        <x:v>8</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K220" s="24" t="n">
-        <x:v>8</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L220" s="28"/>
       <x:c r="M220" s="29"/>
@@ -8372,19 +8370,19 @@
         <x:v>自拼</x:v>
       </x:c>
       <x:c r="B221" s="12" t="str">
-        <x:v>暑_8</x:v>
+        <x:v>暑_9</x:v>
       </x:c>
       <x:c r="C221" s="12" t="str">
-        <x:v>常规外呼</x:v>
+        <x:v>LEC内测</x:v>
       </x:c>
       <x:c r="D221" s="18" t="n">
-        <x:v>29.9</x:v>
+        <x:v>9.9</x:v>
       </x:c>
       <x:c r="E221" s="12" t="str">
-        <x:v>四年级</x:v>
+        <x:v>一年级</x:v>
       </x:c>
       <x:c r="F221" s="21" t="str">
-        <x:v>2026-06-30</x:v>
+        <x:v>2026-07-01</x:v>
       </x:c>
       <x:c r="G221" s="21"/>
       <x:c r="H221" s="21"/>
@@ -8392,10 +8390,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J221" s="24" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K221" s="24" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L221" s="28"/>
       <x:c r="M221" s="29"/>
@@ -8408,7 +8406,7 @@
         <x:v>暑_9</x:v>
       </x:c>
       <x:c r="C222" s="12" t="str">
-        <x:v>LEC内测</x:v>
+        <x:v>WB</x:v>
       </x:c>
       <x:c r="D222" s="18" t="n">
         <x:v>9.9</x:v>
@@ -8417,7 +8415,7 @@
         <x:v>一年级</x:v>
       </x:c>
       <x:c r="F222" s="21" t="str">
-        <x:v>2026-07-01</x:v>
+        <x:v>2026-07-07</x:v>
       </x:c>
       <x:c r="G222" s="21"/>
       <x:c r="H222" s="21"/>
@@ -8425,10 +8423,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J222" s="24" t="n">
-        <x:v>1</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="K222" s="24" t="n">
-        <x:v>1</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="L222" s="28"/>
       <x:c r="M222" s="29"/>
@@ -8447,10 +8445,10 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E223" s="12" t="str">
-        <x:v>一年级</x:v>
+        <x:v>三年级</x:v>
       </x:c>
       <x:c r="F223" s="21" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="G223" s="21"/>
       <x:c r="H223" s="21"/>
@@ -8458,10 +8456,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J223" s="24" t="n">
-        <x:v>192</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="K223" s="24" t="n">
-        <x:v>192</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="L223" s="28"/>
       <x:c r="M223" s="29"/>
@@ -8480,10 +8478,10 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E224" s="12" t="str">
-        <x:v>三年级</x:v>
+        <x:v>四年级</x:v>
       </x:c>
       <x:c r="F224" s="21" t="str">
-        <x:v>2026-07-02</x:v>
+        <x:v>2026-07-07</x:v>
       </x:c>
       <x:c r="G224" s="21"/>
       <x:c r="H224" s="21"/>
@@ -8491,10 +8489,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J224" s="24" t="n">
-        <x:v>89</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="K224" s="24" t="n">
-        <x:v>89</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="L224" s="28"/>
       <x:c r="M224" s="29"/>
@@ -8507,16 +8505,16 @@
         <x:v>暑_9</x:v>
       </x:c>
       <x:c r="C225" s="12" t="str">
-        <x:v>WB</x:v>
+        <x:v>常规外呼</x:v>
       </x:c>
       <x:c r="D225" s="18" t="n">
-        <x:v>9.9</x:v>
+        <x:v>29.9</x:v>
       </x:c>
       <x:c r="E225" s="12" t="str">
-        <x:v>四年级</x:v>
+        <x:v>一年级</x:v>
       </x:c>
       <x:c r="F225" s="21" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
       <x:c r="G225" s="21"/>
       <x:c r="H225" s="21"/>
@@ -8524,10 +8522,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J225" s="24" t="n">
-        <x:v>58</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="K225" s="24" t="n">
-        <x:v>58</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="L225" s="28"/>
       <x:c r="M225" s="29"/>
@@ -8546,7 +8544,7 @@
         <x:v>29.9</x:v>
       </x:c>
       <x:c r="E226" s="12" t="str">
-        <x:v>一年级</x:v>
+        <x:v>三年级</x:v>
       </x:c>
       <x:c r="F226" s="21" t="str">
         <x:v>2026-07-04</x:v>
@@ -8557,10 +8555,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J226" s="24" t="n">
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="K226" s="24" t="n">
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="L226" s="28"/>
       <x:c r="M226" s="29"/>
@@ -8579,10 +8577,10 @@
         <x:v>29.9</x:v>
       </x:c>
       <x:c r="E227" s="12" t="str">
-        <x:v>三年级</x:v>
+        <x:v>四年级</x:v>
       </x:c>
       <x:c r="F227" s="21" t="str">
-        <x:v>2026-07-04</x:v>
+        <x:v>2026-07-07</x:v>
       </x:c>
       <x:c r="G227" s="21"/>
       <x:c r="H227" s="21"/>
@@ -8590,32 +8588,32 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J227" s="24" t="n">
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="K227" s="24" t="n">
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="L227" s="28"/>
       <x:c r="M227" s="29"/>
     </x:row>
     <x:row r="228" ht="15" hidden="0" customHeight="1">
       <x:c r="A228" s="11" t="str">
-        <x:v>自拼</x:v>
+        <x:v>高中</x:v>
       </x:c>
       <x:c r="B228" s="12" t="str">
-        <x:v>暑_9</x:v>
+        <x:v>暑_10</x:v>
       </x:c>
       <x:c r="C228" s="12" t="str">
-        <x:v>常规外呼</x:v>
+        <x:v>AI托管</x:v>
       </x:c>
       <x:c r="D228" s="18" t="n">
-        <x:v>29.9</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E228" s="12" t="str">
-        <x:v>四年级</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F228" s="21" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="G228" s="21"/>
       <x:c r="H228" s="21"/>
@@ -8623,10 +8621,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J228" s="24" t="n">
-        <x:v>18</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="K228" s="24" t="n">
-        <x:v>18</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="L228" s="28"/>
       <x:c r="M228" s="29"/>
@@ -8645,7 +8643,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E229" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F229" s="21" t="str">
         <x:v>2026-06-25</x:v>
@@ -8656,10 +8654,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J229" s="24" t="n">
-        <x:v>55</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="K229" s="24" t="n">
-        <x:v>55</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="L229" s="28"/>
       <x:c r="M229" s="29"/>
@@ -8678,7 +8676,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E230" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F230" s="21" t="str">
         <x:v>2026-06-25</x:v>
@@ -8689,10 +8687,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J230" s="24" t="n">
-        <x:v>115</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="K230" s="24" t="n">
-        <x:v>115</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="L230" s="28"/>
       <x:c r="M230" s="29"/>
@@ -8705,13 +8703,13 @@
         <x:v>暑_10</x:v>
       </x:c>
       <x:c r="C231" s="12" t="str">
-        <x:v>AI托管</x:v>
+        <x:v>LEC内测</x:v>
       </x:c>
       <x:c r="D231" s="18" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E231" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F231" s="21" t="str">
         <x:v>2026-06-25</x:v>
@@ -8722,10 +8720,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J231" s="24" t="n">
-        <x:v>96</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="K231" s="24" t="n">
-        <x:v>96</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="L231" s="28"/>
       <x:c r="M231" s="29"/>
@@ -8744,10 +8742,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E232" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F232" s="21" t="str">
-        <x:v>2026-06-25</x:v>
+        <x:v>2026-06-24</x:v>
       </x:c>
       <x:c r="G232" s="21"/>
       <x:c r="H232" s="21"/>
@@ -8755,10 +8753,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J232" s="24" t="n">
-        <x:v>100</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="K232" s="24" t="n">
-        <x:v>100</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="L232" s="28"/>
       <x:c r="M232" s="29"/>
@@ -8777,10 +8775,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E233" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F233" s="21" t="str">
-        <x:v>2026-06-24</x:v>
+        <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="G233" s="21"/>
       <x:c r="H233" s="21"/>
@@ -8788,10 +8786,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J233" s="24" t="n">
-        <x:v>73</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="K233" s="24" t="n">
-        <x:v>73</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="L233" s="28"/>
       <x:c r="M233" s="29"/>
@@ -8804,16 +8802,16 @@
         <x:v>暑_10</x:v>
       </x:c>
       <x:c r="C234" s="12" t="str">
-        <x:v>LEC内测</x:v>
+        <x:v>LLM外呼</x:v>
       </x:c>
       <x:c r="D234" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>9.9</x:v>
       </x:c>
       <x:c r="E234" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F234" s="21" t="str">
-        <x:v>2026-06-25</x:v>
+        <x:v>2026-06-28</x:v>
       </x:c>
       <x:c r="G234" s="21"/>
       <x:c r="H234" s="21"/>
@@ -8821,10 +8819,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J234" s="24" t="n">
-        <x:v>106</x:v>
+        <x:v>681</x:v>
       </x:c>
       <x:c r="K234" s="24" t="n">
-        <x:v>106</x:v>
+        <x:v>681</x:v>
       </x:c>
       <x:c r="L234" s="28"/>
       <x:c r="M234" s="29"/>
@@ -8843,10 +8841,10 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E235" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F235" s="21" t="str">
-        <x:v>2026-06-28</x:v>
+        <x:v>2026-06-21</x:v>
       </x:c>
       <x:c r="G235" s="21"/>
       <x:c r="H235" s="21"/>
@@ -8854,10 +8852,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J235" s="24" t="n">
-        <x:v>681</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="K235" s="24" t="n">
-        <x:v>681</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="L235" s="28"/>
       <x:c r="M235" s="29"/>
@@ -8870,13 +8868,13 @@
         <x:v>暑_10</x:v>
       </x:c>
       <x:c r="C236" s="12" t="str">
-        <x:v>LLM外呼</x:v>
+        <x:v>外部微转-*</x:v>
       </x:c>
       <x:c r="D236" s="18" t="n">
-        <x:v>9.9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E236" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F236" s="21" t="str">
         <x:v>2026-06-21</x:v>
@@ -8887,10 +8885,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J236" s="24" t="n">
-        <x:v>186</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="K236" s="24" t="n">
-        <x:v>186</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="L236" s="28"/>
       <x:c r="M236" s="29"/>
@@ -8909,7 +8907,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E237" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F237" s="21" t="str">
         <x:v>2026-06-21</x:v>
@@ -8920,10 +8918,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J237" s="24" t="n">
-        <x:v>9</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K237" s="24" t="n">
-        <x:v>9</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L237" s="28"/>
       <x:c r="M237" s="29"/>
@@ -8942,7 +8940,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E238" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F238" s="21" t="str">
         <x:v>2026-06-21</x:v>
@@ -8953,10 +8951,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J238" s="24" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="K238" s="24" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="L238" s="28"/>
       <x:c r="M238" s="29"/>
@@ -8972,13 +8970,13 @@
         <x:v>外部微转-*</x:v>
       </x:c>
       <x:c r="D239" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>28.8</x:v>
       </x:c>
       <x:c r="E239" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F239" s="21" t="str">
-        <x:v>2026-06-21</x:v>
+        <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="G239" s="21"/>
       <x:c r="H239" s="21"/>
@@ -8986,10 +8984,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J239" s="24" t="n">
-        <x:v>6</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="K239" s="24" t="n">
-        <x:v>6</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="L239" s="28"/>
       <x:c r="M239" s="29"/>
@@ -9008,7 +9006,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E240" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F240" s="21" t="str">
         <x:v>2026-06-25</x:v>
@@ -9019,10 +9017,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J240" s="24" t="n">
-        <x:v>357</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="K240" s="24" t="n">
-        <x:v>357</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="L240" s="28"/>
       <x:c r="M240" s="29"/>
@@ -9041,7 +9039,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E241" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F241" s="21" t="str">
         <x:v>2026-06-25</x:v>
@@ -9052,10 +9050,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J241" s="24" t="n">
-        <x:v>291</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="K241" s="24" t="n">
-        <x:v>291</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="L241" s="28"/>
       <x:c r="M241" s="29"/>
@@ -9068,13 +9066,13 @@
         <x:v>暑_10</x:v>
       </x:c>
       <x:c r="C242" s="12" t="str">
-        <x:v>外部微转-*</x:v>
+        <x:v>常规外呼</x:v>
       </x:c>
       <x:c r="D242" s="18" t="n">
-        <x:v>28.8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E242" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F242" s="21" t="str">
         <x:v>2026-06-25</x:v>
@@ -9085,10 +9083,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J242" s="24" t="n">
-        <x:v>320</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="K242" s="24" t="n">
-        <x:v>320</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="L242" s="28"/>
       <x:c r="M242" s="29"/>
@@ -9107,7 +9105,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E243" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F243" s="21" t="str">
         <x:v>2026-06-25</x:v>
@@ -9118,10 +9116,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J243" s="24" t="n">
-        <x:v>697</x:v>
+        <x:v>960</x:v>
       </x:c>
       <x:c r="K243" s="24" t="n">
-        <x:v>697</x:v>
+        <x:v>960</x:v>
       </x:c>
       <x:c r="L243" s="28"/>
       <x:c r="M243" s="29"/>
@@ -9140,7 +9138,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E244" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F244" s="21" t="str">
         <x:v>2026-06-25</x:v>
@@ -9151,10 +9149,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J244" s="24" t="n">
-        <x:v>960</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="K244" s="24" t="n">
-        <x:v>960</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="L244" s="28"/>
       <x:c r="M244" s="29"/>
@@ -9170,10 +9168,10 @@
         <x:v>常规外呼</x:v>
       </x:c>
       <x:c r="D245" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>28.8</x:v>
       </x:c>
       <x:c r="E245" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F245" s="21" t="str">
         <x:v>2026-06-25</x:v>
@@ -9184,10 +9182,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J245" s="24" t="n">
-        <x:v>633</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="K245" s="24" t="n">
-        <x:v>633</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="L245" s="28"/>
       <x:c r="M245" s="29"/>
@@ -9206,7 +9204,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E246" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F246" s="21" t="str">
         <x:v>2026-06-25</x:v>
@@ -9217,10 +9215,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J246" s="24" t="n">
-        <x:v>434</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="K246" s="24" t="n">
-        <x:v>434</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="L246" s="28"/>
       <x:c r="M246" s="29"/>
@@ -9239,7 +9237,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E247" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F247" s="21" t="str">
         <x:v>2026-06-25</x:v>
@@ -9250,10 +9248,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J247" s="24" t="n">
-        <x:v>625</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="K247" s="24" t="n">
-        <x:v>625</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="L247" s="28"/>
       <x:c r="M247" s="29"/>
@@ -9263,33 +9261,41 @@
         <x:v>高中</x:v>
       </x:c>
       <x:c r="B248" s="12" t="str">
-        <x:v>暑_10</x:v>
+        <x:v>暑_11</x:v>
       </x:c>
       <x:c r="C248" s="12" t="str">
-        <x:v>常规外呼</x:v>
+        <x:v>AI托管</x:v>
       </x:c>
       <x:c r="D248" s="18" t="n">
-        <x:v>28.8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E248" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F248" s="21" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="G248" s="21" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="H248" s="21" t="str">
         <x:v>2026-06-25</x:v>
       </x:c>
-      <x:c r="G248" s="21"/>
-      <x:c r="H248" s="21"/>
       <x:c r="I248" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="J248" s="24" t="n">
-        <x:v>558</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="K248" s="24" t="n">
-        <x:v>558</x:v>
-      </x:c>
-      <x:c r="L248" s="28"/>
-      <x:c r="M248" s="29"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L248" s="28" t="n">
+        <x:v>1.0125</x:v>
+      </x:c>
+      <x:c r="M248" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="249" ht="15" hidden="0" customHeight="1">
       <x:c r="A249" s="11" t="str">
@@ -9305,10 +9311,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E249" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F249" s="21" t="str">
-        <x:v>2026-06-30</x:v>
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="G249" s="21" t="str">
         <x:v>2026-07-02</x:v>
@@ -9317,16 +9323,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I249" s="24" t="n">
-        <x:v>80</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="J249" s="24" t="n">
-        <x:v>81</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="K249" s="24" t="n">
-        <x:v>1</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="L249" s="28" t="n">
-        <x:v>1.0125</x:v>
+        <x:v>1.2125</x:v>
       </x:c>
       <x:c r="M249" s="29" t="n">
         <x:v>1</x:v>
@@ -9346,7 +9352,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E250" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F250" s="21" t="str">
         <x:v>2026-07-02</x:v>
@@ -9361,13 +9367,13 @@
         <x:v>160</x:v>
       </x:c>
       <x:c r="J250" s="24" t="n">
-        <x:v>194</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="K250" s="24" t="n">
-        <x:v>34</x:v>
+        <x:v>-21</x:v>
       </x:c>
       <x:c r="L250" s="28" t="n">
-        <x:v>1.2125</x:v>
+        <x:v>0.86875</x:v>
       </x:c>
       <x:c r="M250" s="29" t="n">
         <x:v>1</x:v>
@@ -9381,16 +9387,16 @@
         <x:v>暑_11</x:v>
       </x:c>
       <x:c r="C251" s="12" t="str">
-        <x:v>AI托管</x:v>
+        <x:v>LLM外呼</x:v>
       </x:c>
       <x:c r="D251" s="18" t="n">
-        <x:v>0</x:v>
+        <x:v>9.9</x:v>
       </x:c>
       <x:c r="E251" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F251" s="21" t="str">
-        <x:v>2026-07-02</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
       <x:c r="G251" s="21" t="str">
         <x:v>2026-07-02</x:v>
@@ -9399,16 +9405,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I251" s="24" t="n">
-        <x:v>160</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="J251" s="24" t="n">
-        <x:v>139</x:v>
+        <x:v>883</x:v>
       </x:c>
       <x:c r="K251" s="24" t="n">
-        <x:v>-21</x:v>
+        <x:v>833</x:v>
       </x:c>
       <x:c r="L251" s="28" t="n">
-        <x:v>0.86875</x:v>
+        <x:v>17.66</x:v>
       </x:c>
       <x:c r="M251" s="29" t="n">
         <x:v>1</x:v>
@@ -9428,10 +9434,10 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E252" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F252" s="21" t="str">
-        <x:v>2026-07-04</x:v>
+        <x:v>2026-07-05</x:v>
       </x:c>
       <x:c r="G252" s="21" t="str">
         <x:v>2026-07-02</x:v>
@@ -9440,16 +9446,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I252" s="24" t="n">
-        <x:v>50</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="J252" s="24" t="n">
-        <x:v>883</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="K252" s="24" t="n">
-        <x:v>833</x:v>
+        <x:v>-671</x:v>
       </x:c>
       <x:c r="L252" s="28" t="n">
-        <x:v>17.66</x:v>
+        <x:v>0.2544444444444444</x:v>
       </x:c>
       <x:c r="M252" s="29" t="n">
         <x:v>1</x:v>
@@ -9469,7 +9475,7 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E253" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F253" s="21" t="str">
         <x:v>2026-07-05</x:v>
@@ -9481,16 +9487,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I253" s="24" t="n">
-        <x:v>900</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="J253" s="24" t="n">
-        <x:v>229</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K253" s="24" t="n">
-        <x:v>-671</x:v>
+        <x:v>-198</x:v>
       </x:c>
       <x:c r="L253" s="28" t="n">
-        <x:v>0.2544444444444444</x:v>
+        <x:v>0.01</x:v>
       </x:c>
       <x:c r="M253" s="29" t="n">
         <x:v>1</x:v>
@@ -9504,16 +9510,16 @@
         <x:v>暑_11</x:v>
       </x:c>
       <x:c r="C254" s="12" t="str">
-        <x:v>LLM外呼</x:v>
+        <x:v>图书店铺</x:v>
       </x:c>
       <x:c r="D254" s="18" t="n">
-        <x:v>9.9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E254" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F254" s="21" t="str">
-        <x:v>2026-07-05</x:v>
+        <x:v>2026-06-30</x:v>
       </x:c>
       <x:c r="G254" s="21" t="str">
         <x:v>2026-07-02</x:v>
@@ -9522,16 +9528,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I254" s="24" t="n">
-        <x:v>200</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="J254" s="24" t="n">
-        <x:v>2</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="K254" s="24" t="n">
-        <x:v>-198</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="L254" s="28" t="n">
-        <x:v>0.01</x:v>
+        <x:v>1.29</x:v>
       </x:c>
       <x:c r="M254" s="29" t="n">
         <x:v>1</x:v>
@@ -9551,10 +9557,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E255" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F255" s="21" t="str">
-        <x:v>2026-06-30</x:v>
+        <x:v>2026-07-01</x:v>
       </x:c>
       <x:c r="G255" s="21" t="str">
         <x:v>2026-07-02</x:v>
@@ -9563,16 +9569,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I255" s="24" t="n">
-        <x:v>100</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="J255" s="24" t="n">
-        <x:v>129</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="K255" s="24" t="n">
-        <x:v>29</x:v>
+        <x:v>-111</x:v>
       </x:c>
       <x:c r="L255" s="28" t="n">
-        <x:v>1.29</x:v>
+        <x:v>0.26</x:v>
       </x:c>
       <x:c r="M255" s="29" t="n">
         <x:v>1</x:v>
@@ -9592,10 +9598,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E256" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F256" s="21" t="str">
-        <x:v>2026-07-01</x:v>
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="G256" s="21" t="str">
         <x:v>2026-07-02</x:v>
@@ -9607,13 +9613,13 @@
         <x:v>150</x:v>
       </x:c>
       <x:c r="J256" s="24" t="n">
-        <x:v>39</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="K256" s="24" t="n">
-        <x:v>-111</x:v>
+        <x:v>-121</x:v>
       </x:c>
       <x:c r="L256" s="28" t="n">
-        <x:v>0.26</x:v>
+        <x:v>0.19333333333333333</x:v>
       </x:c>
       <x:c r="M256" s="29" t="n">
         <x:v>1</x:v>
@@ -9627,17 +9633,15 @@
         <x:v>暑_11</x:v>
       </x:c>
       <x:c r="C257" s="12" t="str">
-        <x:v>图书店铺</x:v>
+        <x:v>外部微转-*</x:v>
       </x:c>
       <x:c r="D257" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E257" s="12" t="str">
-        <x:v>高三</x:v>
-      </x:c>
-      <x:c r="F257" s="21" t="str">
-        <x:v>2026-07-02</x:v>
-      </x:c>
+        <x:v>高一</x:v>
+      </x:c>
+      <x:c r="F257" s="21"/>
       <x:c r="G257" s="21" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
@@ -9648,13 +9652,13 @@
         <x:v>150</x:v>
       </x:c>
       <x:c r="J257" s="24" t="n">
-        <x:v>29</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K257" s="24" t="n">
-        <x:v>-121</x:v>
+        <x:v>-150</x:v>
       </x:c>
       <x:c r="L257" s="28" t="n">
-        <x:v>0.19333333333333333</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M257" s="29" t="n">
         <x:v>1</x:v>
@@ -9674,7 +9678,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E258" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F258" s="21"/>
       <x:c r="G258" s="21" t="str">
@@ -9684,13 +9688,13 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I258" s="24" t="n">
-        <x:v>150</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="J258" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K258" s="24" t="n">
-        <x:v>-150</x:v>
+        <x:v>-200</x:v>
       </x:c>
       <x:c r="L258" s="28" t="n">
         <x:v>0</x:v>
@@ -9713,7 +9717,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E259" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F259" s="21"/>
       <x:c r="G259" s="21" t="str">
@@ -9723,13 +9727,13 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I259" s="24" t="n">
-        <x:v>200</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="J259" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K259" s="24" t="n">
-        <x:v>-200</x:v>
+        <x:v>-150</x:v>
       </x:c>
       <x:c r="L259" s="28" t="n">
         <x:v>0</x:v>
@@ -9749,12 +9753,14 @@
         <x:v>外部微转-*</x:v>
       </x:c>
       <x:c r="D260" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>28.8</x:v>
       </x:c>
       <x:c r="E260" s="12" t="str">
-        <x:v>高三</x:v>
-      </x:c>
-      <x:c r="F260" s="21"/>
+        <x:v>高一</x:v>
+      </x:c>
+      <x:c r="F260" s="21" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
       <x:c r="G260" s="21" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
@@ -9762,16 +9768,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I260" s="24" t="n">
-        <x:v>150</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="J260" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="K260" s="24" t="n">
-        <x:v>-150</x:v>
+        <x:v>-2</x:v>
       </x:c>
       <x:c r="L260" s="28" t="n">
-        <x:v>0</x:v>
+        <x:v>0.9933333333333333</x:v>
       </x:c>
       <x:c r="M260" s="29" t="n">
         <x:v>1</x:v>
@@ -9791,10 +9797,10 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E261" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F261" s="21" t="str">
-        <x:v>2026-06-30</x:v>
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="G261" s="21" t="str">
         <x:v>2026-07-02</x:v>
@@ -9803,16 +9809,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I261" s="24" t="n">
-        <x:v>300</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="J261" s="24" t="n">
-        <x:v>298</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="K261" s="24" t="n">
-        <x:v>-2</x:v>
+        <x:v>-156</x:v>
       </x:c>
       <x:c r="L261" s="28" t="n">
-        <x:v>0.9933333333333333</x:v>
+        <x:v>0.7056603773584905</x:v>
       </x:c>
       <x:c r="M261" s="29" t="n">
         <x:v>1</x:v>
@@ -9832,7 +9838,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E262" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F262" s="21" t="str">
         <x:v>2026-07-02</x:v>
@@ -9844,16 +9850,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I262" s="24" t="n">
-        <x:v>530</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="J262" s="24" t="n">
-        <x:v>374</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="K262" s="24" t="n">
-        <x:v>-156</x:v>
+        <x:v>-115</x:v>
       </x:c>
       <x:c r="L262" s="28" t="n">
-        <x:v>0.7056603773584905</x:v>
+        <x:v>0.8083333333333333</x:v>
       </x:c>
       <x:c r="M262" s="29" t="n">
         <x:v>1</x:v>
@@ -9867,13 +9873,13 @@
         <x:v>暑_11</x:v>
       </x:c>
       <x:c r="C263" s="12" t="str">
-        <x:v>外部微转-*</x:v>
+        <x:v>常规外呼</x:v>
       </x:c>
       <x:c r="D263" s="18" t="n">
-        <x:v>28.8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E263" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F263" s="21" t="str">
         <x:v>2026-07-02</x:v>
@@ -9885,16 +9891,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I263" s="24" t="n">
-        <x:v>600</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="J263" s="24" t="n">
-        <x:v>485</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="K263" s="24" t="n">
-        <x:v>-115</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="L263" s="28" t="n">
-        <x:v>0.8083333333333333</x:v>
+        <x:v>1.7055555555555555</x:v>
       </x:c>
       <x:c r="M263" s="29" t="n">
         <x:v>1</x:v>
@@ -9914,7 +9920,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E264" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F264" s="21" t="str">
         <x:v>2026-07-02</x:v>
@@ -9926,16 +9932,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I264" s="24" t="n">
-        <x:v>180</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="J264" s="24" t="n">
-        <x:v>307</x:v>
+        <x:v>1313</x:v>
       </x:c>
       <x:c r="K264" s="24" t="n">
-        <x:v>127</x:v>
+        <x:v>-187</x:v>
       </x:c>
       <x:c r="L264" s="28" t="n">
-        <x:v>1.7055555555555555</x:v>
+        <x:v>0.8753333333333333</x:v>
       </x:c>
       <x:c r="M264" s="29" t="n">
         <x:v>1</x:v>
@@ -9955,7 +9961,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E265" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F265" s="21" t="str">
         <x:v>2026-07-02</x:v>
@@ -9967,16 +9973,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I265" s="24" t="n">
-        <x:v>1500</x:v>
+        <x:v>870</x:v>
       </x:c>
       <x:c r="J265" s="24" t="n">
-        <x:v>1313</x:v>
+        <x:v>854</x:v>
       </x:c>
       <x:c r="K265" s="24" t="n">
-        <x:v>-187</x:v>
+        <x:v>-16</x:v>
       </x:c>
       <x:c r="L265" s="28" t="n">
-        <x:v>0.8753333333333333</x:v>
+        <x:v>0.9816091954022989</x:v>
       </x:c>
       <x:c r="M265" s="29" t="n">
         <x:v>1</x:v>
@@ -9993,35 +9999,27 @@
         <x:v>常规外呼</x:v>
       </x:c>
       <x:c r="D266" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>9.9</x:v>
       </x:c>
       <x:c r="E266" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F266" s="21" t="str">
-        <x:v>2026-07-02</x:v>
-      </x:c>
-      <x:c r="G266" s="21" t="str">
-        <x:v>2026-07-02</x:v>
-      </x:c>
-      <x:c r="H266" s="21" t="str">
-        <x:v>2026-06-25</x:v>
-      </x:c>
+        <x:v>2026-06-28</x:v>
+      </x:c>
+      <x:c r="G266" s="21"/>
+      <x:c r="H266" s="21"/>
       <x:c r="I266" s="24" t="n">
-        <x:v>870</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J266" s="24" t="n">
-        <x:v>854</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K266" s="24" t="n">
-        <x:v>-16</x:v>
-      </x:c>
-      <x:c r="L266" s="28" t="n">
-        <x:v>0.9816091954022989</x:v>
-      </x:c>
-      <x:c r="M266" s="29" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="L266" s="28"/>
+      <x:c r="M266" s="29"/>
     </x:row>
     <x:row r="267" ht="15" hidden="0" customHeight="1">
       <x:c r="A267" s="11" t="str">
@@ -10037,7 +10035,7 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E267" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F267" s="21" t="str">
         <x:v>2026-06-28</x:v>
@@ -10048,10 +10046,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J267" s="24" t="n">
-        <x:v>5</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="K267" s="24" t="n">
-        <x:v>5</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="L267" s="28"/>
       <x:c r="M267" s="29"/>
@@ -10070,7 +10068,7 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E268" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F268" s="21" t="str">
         <x:v>2026-06-28</x:v>
@@ -10081,10 +10079,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J268" s="24" t="n">
-        <x:v>63</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="K268" s="24" t="n">
-        <x:v>63</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="L268" s="28"/>
       <x:c r="M268" s="29"/>
@@ -10100,27 +10098,31 @@
         <x:v>常规外呼</x:v>
       </x:c>
       <x:c r="D269" s="18" t="n">
-        <x:v>9.9</x:v>
+        <x:v>28.8</x:v>
       </x:c>
       <x:c r="E269" s="12" t="str">
-        <x:v>高三</x:v>
-      </x:c>
-      <x:c r="F269" s="21" t="str">
-        <x:v>2026-06-28</x:v>
-      </x:c>
-      <x:c r="G269" s="21"/>
-      <x:c r="H269" s="21"/>
+        <x:v>高一</x:v>
+      </x:c>
+      <x:c r="F269" s="21"/>
+      <x:c r="G269" s="21" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="H269" s="21" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
       <x:c r="I269" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J269" s="24" t="n">
-        <x:v>10</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K269" s="24" t="n">
-        <x:v>10</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L269" s="28"/>
-      <x:c r="M269" s="29"/>
+      <x:c r="M269" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="270" ht="15" hidden="0" customHeight="1">
       <x:c r="A270" s="11" t="str">
@@ -10136,9 +10138,11 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E270" s="12" t="str">
-        <x:v>高一</x:v>
-      </x:c>
-      <x:c r="F270" s="21"/>
+        <x:v>高二</x:v>
+      </x:c>
+      <x:c r="F270" s="21" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
       <x:c r="G270" s="21" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
@@ -10146,15 +10150,17 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I270" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="J270" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>788</x:v>
       </x:c>
       <x:c r="K270" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L270" s="28"/>
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="L270" s="28" t="n">
+        <x:v>1.1257142857142857</x:v>
+      </x:c>
       <x:c r="M270" s="29" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -10173,7 +10179,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E271" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F271" s="21" t="str">
         <x:v>2026-07-02</x:v>
@@ -10185,16 +10191,16 @@
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="I271" s="24" t="n">
-        <x:v>700</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="J271" s="24" t="n">
-        <x:v>788</x:v>
+        <x:v>731</x:v>
       </x:c>
       <x:c r="K271" s="24" t="n">
-        <x:v>88</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="L271" s="28" t="n">
-        <x:v>1.1257142857142857</x:v>
+        <x:v>1.1246153846153846</x:v>
       </x:c>
       <x:c r="M271" s="29" t="n">
         <x:v>1</x:v>
@@ -10205,40 +10211,40 @@
         <x:v>高中</x:v>
       </x:c>
       <x:c r="B272" s="12" t="str">
-        <x:v>暑_11</x:v>
+        <x:v>暑_12</x:v>
       </x:c>
       <x:c r="C272" s="12" t="str">
-        <x:v>常规外呼</x:v>
+        <x:v>AI托管</x:v>
       </x:c>
       <x:c r="D272" s="18" t="n">
-        <x:v>28.8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E272" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F272" s="21" t="str">
+        <x:v>2026-07-07</x:v>
+      </x:c>
+      <x:c r="G272" s="21" t="str">
+        <x:v>2026-07-09</x:v>
+      </x:c>
+      <x:c r="H272" s="21" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
-      <x:c r="G272" s="21" t="str">
-        <x:v>2026-07-02</x:v>
-      </x:c>
-      <x:c r="H272" s="21" t="str">
-        <x:v>2026-06-25</x:v>
-      </x:c>
       <x:c r="I272" s="24" t="n">
-        <x:v>650</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="J272" s="24" t="n">
-        <x:v>731</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="K272" s="24" t="n">
-        <x:v>81</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="L272" s="28" t="n">
-        <x:v>1.1246153846153846</x:v>
+        <x:v>1.3857142857142857</x:v>
       </x:c>
       <x:c r="M272" s="29" t="n">
-        <x:v>1</x:v>
+        <x:v>0.8333333333333334</x:v>
       </x:c>
     </x:row>
     <x:row r="273" ht="15" hidden="0" customHeight="1">
@@ -10255,7 +10261,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E273" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F273" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -10267,16 +10273,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I273" s="24" t="n">
-        <x:v>70</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="J273" s="24" t="n">
-        <x:v>97</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="K273" s="24" t="n">
-        <x:v>27</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="L273" s="28" t="n">
-        <x:v>1.3857142857142857</x:v>
+        <x:v>1.1285714285714286</x:v>
       </x:c>
       <x:c r="M273" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -10296,7 +10302,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E274" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F274" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -10311,13 +10317,13 @@
         <x:v>140</x:v>
       </x:c>
       <x:c r="J274" s="24" t="n">
-        <x:v>158</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="K274" s="24" t="n">
-        <x:v>18</x:v>
+        <x:v>-39</x:v>
       </x:c>
       <x:c r="L274" s="28" t="n">
-        <x:v>1.1285714285714286</x:v>
+        <x:v>0.7214285714285714</x:v>
       </x:c>
       <x:c r="M274" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -10331,16 +10337,16 @@
         <x:v>暑_12</x:v>
       </x:c>
       <x:c r="C275" s="12" t="str">
-        <x:v>AI托管</x:v>
+        <x:v>LLM外呼</x:v>
       </x:c>
       <x:c r="D275" s="18" t="n">
-        <x:v>0</x:v>
+        <x:v>9.9</x:v>
       </x:c>
       <x:c r="E275" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F275" s="21" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
       <x:c r="G275" s="21" t="str">
         <x:v>2026-07-09</x:v>
@@ -10349,16 +10355,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I275" s="24" t="n">
-        <x:v>140</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="J275" s="24" t="n">
-        <x:v>101</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="K275" s="24" t="n">
-        <x:v>-39</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="L275" s="28" t="n">
-        <x:v>0.7214285714285714</x:v>
+        <x:v>3.4</x:v>
       </x:c>
       <x:c r="M275" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -10378,10 +10384,10 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E276" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F276" s="21" t="str">
-        <x:v>2026-07-04</x:v>
+        <x:v>2026-07-07</x:v>
       </x:c>
       <x:c r="G276" s="21" t="str">
         <x:v>2026-07-09</x:v>
@@ -10390,16 +10396,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I276" s="24" t="n">
-        <x:v>100</x:v>
+        <x:v>800</x:v>
       </x:c>
       <x:c r="J276" s="24" t="n">
-        <x:v>340</x:v>
+        <x:v>787</x:v>
       </x:c>
       <x:c r="K276" s="24" t="n">
-        <x:v>240</x:v>
+        <x:v>-13</x:v>
       </x:c>
       <x:c r="L276" s="28" t="n">
-        <x:v>3.4</x:v>
+        <x:v>0.98375</x:v>
       </x:c>
       <x:c r="M276" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -10419,10 +10425,10 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E277" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F277" s="21" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-07-05</x:v>
       </x:c>
       <x:c r="G277" s="21" t="str">
         <x:v>2026-07-09</x:v>
@@ -10431,16 +10437,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I277" s="24" t="n">
-        <x:v>800</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="J277" s="24" t="n">
-        <x:v>787</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="K277" s="24" t="n">
-        <x:v>-13</x:v>
+        <x:v>-233</x:v>
       </x:c>
       <x:c r="L277" s="28" t="n">
-        <x:v>0.98375</x:v>
+        <x:v>0.6671428571428571</x:v>
       </x:c>
       <x:c r="M277" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -10454,17 +10460,15 @@
         <x:v>暑_12</x:v>
       </x:c>
       <x:c r="C278" s="12" t="str">
-        <x:v>LLM外呼</x:v>
+        <x:v>外部微转-*</x:v>
       </x:c>
       <x:c r="D278" s="18" t="n">
-        <x:v>9.9</x:v>
+        <x:v>28.8</x:v>
       </x:c>
       <x:c r="E278" s="12" t="str">
-        <x:v>高三</x:v>
-      </x:c>
-      <x:c r="F278" s="21" t="str">
-        <x:v>2026-07-05</x:v>
-      </x:c>
+        <x:v>高一</x:v>
+      </x:c>
+      <x:c r="F278" s="21"/>
       <x:c r="G278" s="21" t="str">
         <x:v>2026-07-09</x:v>
       </x:c>
@@ -10472,17 +10476,15 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I278" s="24" t="n">
-        <x:v>700</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J278" s="24" t="n">
-        <x:v>467</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K278" s="24" t="n">
-        <x:v>-233</x:v>
-      </x:c>
-      <x:c r="L278" s="28" t="n">
-        <x:v>0.6671428571428571</x:v>
-      </x:c>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L278" s="28"/>
       <x:c r="M278" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
       </x:c>
@@ -10501,9 +10503,11 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E279" s="12" t="str">
-        <x:v>高一</x:v>
-      </x:c>
-      <x:c r="F279" s="21"/>
+        <x:v>高二</x:v>
+      </x:c>
+      <x:c r="F279" s="21" t="str">
+        <x:v>2026-07-07</x:v>
+      </x:c>
       <x:c r="G279" s="21" t="str">
         <x:v>2026-07-09</x:v>
       </x:c>
@@ -10511,15 +10515,17 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I279" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="J279" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K279" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L279" s="28"/>
+      <x:c r="L279" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="M279" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
       </x:c>
@@ -10538,7 +10544,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E280" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F280" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -10550,16 +10556,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I280" s="24" t="n">
-        <x:v>150</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="J280" s="24" t="n">
-        <x:v>150</x:v>
+        <x:v>397</x:v>
       </x:c>
       <x:c r="K280" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>-88</x:v>
       </x:c>
       <x:c r="L280" s="28" t="n">
-        <x:v>1</x:v>
+        <x:v>0.8185567010309278</x:v>
       </x:c>
       <x:c r="M280" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -10573,13 +10579,13 @@
         <x:v>暑_12</x:v>
       </x:c>
       <x:c r="C281" s="12" t="str">
-        <x:v>外部微转-*</x:v>
+        <x:v>常规外呼</x:v>
       </x:c>
       <x:c r="D281" s="18" t="n">
-        <x:v>28.8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E281" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F281" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -10591,16 +10597,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I281" s="24" t="n">
-        <x:v>485</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="J281" s="24" t="n">
-        <x:v>397</x:v>
+        <x:v>303</x:v>
       </x:c>
       <x:c r="K281" s="24" t="n">
-        <x:v>-88</x:v>
+        <x:v>-32</x:v>
       </x:c>
       <x:c r="L281" s="28" t="n">
-        <x:v>0.8185567010309278</x:v>
+        <x:v>0.9044776119402985</x:v>
       </x:c>
       <x:c r="M281" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -10620,7 +10626,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E282" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F282" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -10632,16 +10638,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I282" s="24" t="n">
-        <x:v>335</x:v>
+        <x:v>980</x:v>
       </x:c>
       <x:c r="J282" s="24" t="n">
-        <x:v>303</x:v>
+        <x:v>807</x:v>
       </x:c>
       <x:c r="K282" s="24" t="n">
-        <x:v>-32</x:v>
+        <x:v>-173</x:v>
       </x:c>
       <x:c r="L282" s="28" t="n">
-        <x:v>0.9044776119402985</x:v>
+        <x:v>0.823469387755102</x:v>
       </x:c>
       <x:c r="M282" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -10661,7 +10667,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E283" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F283" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -10673,16 +10679,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I283" s="24" t="n">
-        <x:v>980</x:v>
+        <x:v>1240</x:v>
       </x:c>
       <x:c r="J283" s="24" t="n">
-        <x:v>807</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="K283" s="24" t="n">
-        <x:v>-173</x:v>
+        <x:v>-538</x:v>
       </x:c>
       <x:c r="L283" s="28" t="n">
-        <x:v>0.823469387755102</x:v>
+        <x:v>0.5661290322580645</x:v>
       </x:c>
       <x:c r="M283" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -10699,13 +10705,13 @@
         <x:v>常规外呼</x:v>
       </x:c>
       <x:c r="D284" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>28.8</x:v>
       </x:c>
       <x:c r="E284" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F284" s="21" t="str">
-        <x:v>2026-07-07</x:v>
+        <x:v>2026-07-03</x:v>
       </x:c>
       <x:c r="G284" s="21" t="str">
         <x:v>2026-07-09</x:v>
@@ -10714,17 +10720,15 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I284" s="24" t="n">
-        <x:v>1240</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J284" s="24" t="n">
-        <x:v>702</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K284" s="24" t="n">
-        <x:v>-538</x:v>
-      </x:c>
-      <x:c r="L284" s="28" t="n">
-        <x:v>0.5661290322580645</x:v>
-      </x:c>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L284" s="28"/>
       <x:c r="M284" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
       </x:c>
@@ -10743,10 +10747,10 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E285" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F285" s="21" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-07</x:v>
       </x:c>
       <x:c r="G285" s="21" t="str">
         <x:v>2026-07-09</x:v>
@@ -10755,15 +10759,17 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I285" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="J285" s="24" t="n">
-        <x:v>1</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="K285" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L285" s="28"/>
+        <x:v>-30</x:v>
+      </x:c>
+      <x:c r="L285" s="28" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
       <x:c r="M285" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
       </x:c>
@@ -10782,7 +10788,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E286" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F286" s="21" t="str">
         <x:v>2026-07-07</x:v>
@@ -10794,16 +10800,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="I286" s="24" t="n">
-        <x:v>300</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="J286" s="24" t="n">
-        <x:v>270</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="K286" s="24" t="n">
-        <x:v>-30</x:v>
+        <x:v>-68</x:v>
       </x:c>
       <x:c r="L286" s="28" t="n">
-        <x:v>0.9</x:v>
+        <x:v>0.864</x:v>
       </x:c>
       <x:c r="M286" s="29" t="n">
         <x:v>0.8333333333333334</x:v>
@@ -10814,48 +10820,40 @@
         <x:v>高中</x:v>
       </x:c>
       <x:c r="B287" s="12" t="str">
-        <x:v>暑_12</x:v>
+        <x:v>暑_7</x:v>
       </x:c>
       <x:c r="C287" s="12" t="str">
-        <x:v>常规外呼</x:v>
+        <x:v>LLM外呼</x:v>
       </x:c>
       <x:c r="D287" s="18" t="n">
-        <x:v>28.8</x:v>
+        <x:v>9.9</x:v>
       </x:c>
       <x:c r="E287" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F287" s="21" t="str">
-        <x:v>2026-07-07</x:v>
-      </x:c>
-      <x:c r="G287" s="21" t="str">
-        <x:v>2026-07-09</x:v>
-      </x:c>
-      <x:c r="H287" s="21" t="str">
-        <x:v>2026-07-02</x:v>
-      </x:c>
+        <x:v>2026-06-21</x:v>
+      </x:c>
+      <x:c r="G287" s="21"/>
+      <x:c r="H287" s="21"/>
       <x:c r="I287" s="24" t="n">
-        <x:v>500</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J287" s="24" t="n">
-        <x:v>432</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K287" s="24" t="n">
-        <x:v>-68</x:v>
-      </x:c>
-      <x:c r="L287" s="28" t="n">
-        <x:v>0.864</x:v>
-      </x:c>
-      <x:c r="M287" s="29" t="n">
-        <x:v>0.8333333333333334</x:v>
-      </x:c>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L287" s="28"/>
+      <x:c r="M287" s="29"/>
     </x:row>
     <x:row r="288" ht="15" hidden="0" customHeight="1">
       <x:c r="A288" s="11" t="str">
         <x:v>高中</x:v>
       </x:c>
       <x:c r="B288" s="12" t="str">
-        <x:v>暑_7</x:v>
+        <x:v>暑_8</x:v>
       </x:c>
       <x:c r="C288" s="12" t="str">
         <x:v>LLM外呼</x:v>
@@ -10867,7 +10865,7 @@
         <x:v>高一</x:v>
       </x:c>
       <x:c r="F288" s="21" t="str">
-        <x:v>2026-06-21</x:v>
+        <x:v>2026-06-28</x:v>
       </x:c>
       <x:c r="G288" s="21"/>
       <x:c r="H288" s="21"/>
@@ -10875,10 +10873,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J288" s="24" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="K288" s="24" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="L288" s="28"/>
       <x:c r="M288" s="29"/>
@@ -10897,7 +10895,7 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E289" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F289" s="21" t="str">
         <x:v>2026-06-28</x:v>
@@ -10908,10 +10906,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J289" s="24" t="n">
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K289" s="24" t="n">
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L289" s="28"/>
       <x:c r="M289" s="29"/>
@@ -10921,19 +10919,19 @@
         <x:v>高中</x:v>
       </x:c>
       <x:c r="B290" s="12" t="str">
-        <x:v>暑_8</x:v>
+        <x:v>暑_9</x:v>
       </x:c>
       <x:c r="C290" s="12" t="str">
-        <x:v>LLM外呼</x:v>
+        <x:v>AI托管</x:v>
       </x:c>
       <x:c r="D290" s="18" t="n">
-        <x:v>9.9</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E290" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F290" s="21" t="str">
-        <x:v>2026-06-28</x:v>
+        <x:v>2026-06-18</x:v>
       </x:c>
       <x:c r="G290" s="21"/>
       <x:c r="H290" s="21"/>
@@ -10941,10 +10939,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J290" s="24" t="n">
-        <x:v>1</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="K290" s="24" t="n">
-        <x:v>1</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="L290" s="28"/>
       <x:c r="M290" s="29"/>
@@ -10963,7 +10961,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E291" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F291" s="21" t="str">
         <x:v>2026-06-18</x:v>
@@ -10974,10 +10972,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J291" s="24" t="n">
-        <x:v>27</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="K291" s="24" t="n">
-        <x:v>27</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="L291" s="28"/>
       <x:c r="M291" s="29"/>
@@ -10996,7 +10994,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E292" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F292" s="21" t="str">
         <x:v>2026-06-18</x:v>
@@ -11007,10 +11005,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J292" s="24" t="n">
-        <x:v>63</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="K292" s="24" t="n">
-        <x:v>63</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="L292" s="28"/>
       <x:c r="M292" s="29"/>
@@ -11023,13 +11021,13 @@
         <x:v>暑_9</x:v>
       </x:c>
       <x:c r="C293" s="12" t="str">
-        <x:v>AI托管</x:v>
+        <x:v>LEC内测</x:v>
       </x:c>
       <x:c r="D293" s="18" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E293" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F293" s="21" t="str">
         <x:v>2026-06-18</x:v>
@@ -11040,10 +11038,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J293" s="24" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="K293" s="24" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="L293" s="28"/>
       <x:c r="M293" s="29"/>
@@ -11062,7 +11060,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E294" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F294" s="21" t="str">
         <x:v>2026-06-18</x:v>
@@ -11073,10 +11071,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J294" s="24" t="n">
-        <x:v>10</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K294" s="24" t="n">
-        <x:v>10</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L294" s="28"/>
       <x:c r="M294" s="29"/>
@@ -11095,10 +11093,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E295" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F295" s="21" t="str">
-        <x:v>2026-06-18</x:v>
+        <x:v>2026-06-17</x:v>
       </x:c>
       <x:c r="G295" s="21"/>
       <x:c r="H295" s="21"/>
@@ -11106,10 +11104,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J295" s="24" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K295" s="24" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L295" s="28"/>
       <x:c r="M295" s="29"/>
@@ -11122,16 +11120,16 @@
         <x:v>暑_9</x:v>
       </x:c>
       <x:c r="C296" s="12" t="str">
-        <x:v>LEC内测</x:v>
+        <x:v>LLM外呼</x:v>
       </x:c>
       <x:c r="D296" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>9.9</x:v>
       </x:c>
       <x:c r="E296" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F296" s="21" t="str">
-        <x:v>2026-06-17</x:v>
+        <x:v>2026-06-20</x:v>
       </x:c>
       <x:c r="G296" s="21"/>
       <x:c r="H296" s="21"/>
@@ -11139,10 +11137,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J296" s="24" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K296" s="24" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L296" s="28"/>
       <x:c r="M296" s="29"/>
@@ -11161,10 +11159,10 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E297" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F297" s="21" t="str">
-        <x:v>2026-06-20</x:v>
+        <x:v>2026-07-05</x:v>
       </x:c>
       <x:c r="G297" s="21"/>
       <x:c r="H297" s="21"/>
@@ -11172,10 +11170,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J297" s="24" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="K297" s="24" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="L297" s="28"/>
       <x:c r="M297" s="29"/>
@@ -11194,7 +11192,7 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="E298" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F298" s="21" t="str">
         <x:v>2026-07-05</x:v>
@@ -11205,10 +11203,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J298" s="24" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K298" s="24" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L298" s="28"/>
       <x:c r="M298" s="29"/>
@@ -11221,16 +11219,16 @@
         <x:v>暑_9</x:v>
       </x:c>
       <x:c r="C299" s="12" t="str">
-        <x:v>LLM外呼</x:v>
+        <x:v>外部微转-*</x:v>
       </x:c>
       <x:c r="D299" s="18" t="n">
-        <x:v>9.9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E299" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F299" s="21" t="str">
-        <x:v>2026-07-05</x:v>
+        <x:v>2026-06-18</x:v>
       </x:c>
       <x:c r="G299" s="21"/>
       <x:c r="H299" s="21"/>
@@ -11238,10 +11236,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J299" s="24" t="n">
-        <x:v>2</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="K299" s="24" t="n">
-        <x:v>2</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="L299" s="28"/>
       <x:c r="M299" s="29"/>
@@ -11260,7 +11258,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E300" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F300" s="21" t="str">
         <x:v>2026-06-18</x:v>
@@ -11271,10 +11269,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J300" s="24" t="n">
-        <x:v>146</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="K300" s="24" t="n">
-        <x:v>146</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="L300" s="28"/>
       <x:c r="M300" s="29"/>
@@ -11293,7 +11291,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E301" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F301" s="21" t="str">
         <x:v>2026-06-18</x:v>
@@ -11304,10 +11302,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J301" s="24" t="n">
-        <x:v>157</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="K301" s="24" t="n">
-        <x:v>157</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="L301" s="28"/>
       <x:c r="M301" s="29"/>
@@ -11323,10 +11321,10 @@
         <x:v>外部微转-*</x:v>
       </x:c>
       <x:c r="D302" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>28.8</x:v>
       </x:c>
       <x:c r="E302" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F302" s="21" t="str">
         <x:v>2026-06-18</x:v>
@@ -11337,10 +11335,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J302" s="24" t="n">
-        <x:v>136</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="K302" s="24" t="n">
-        <x:v>136</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="L302" s="28"/>
       <x:c r="M302" s="29"/>
@@ -11359,10 +11357,10 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E303" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F303" s="21" t="str">
-        <x:v>2026-06-18</x:v>
+        <x:v>2026-06-17</x:v>
       </x:c>
       <x:c r="G303" s="21"/>
       <x:c r="H303" s="21"/>
@@ -11370,10 +11368,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J303" s="24" t="n">
-        <x:v>51</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="K303" s="24" t="n">
-        <x:v>51</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="L303" s="28"/>
       <x:c r="M303" s="29"/>
@@ -11392,10 +11390,10 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E304" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F304" s="21" t="str">
-        <x:v>2026-06-17</x:v>
+        <x:v>2026-06-18</x:v>
       </x:c>
       <x:c r="G304" s="21"/>
       <x:c r="H304" s="21"/>
@@ -11403,10 +11401,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J304" s="24" t="n">
-        <x:v>17</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="K304" s="24" t="n">
-        <x:v>17</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="L304" s="28"/>
       <x:c r="M304" s="29"/>
@@ -11419,13 +11417,13 @@
         <x:v>暑_9</x:v>
       </x:c>
       <x:c r="C305" s="12" t="str">
-        <x:v>外部微转-*</x:v>
+        <x:v>常规外呼</x:v>
       </x:c>
       <x:c r="D305" s="18" t="n">
-        <x:v>28.8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E305" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F305" s="21" t="str">
         <x:v>2026-06-18</x:v>
@@ -11436,10 +11434,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J305" s="24" t="n">
-        <x:v>30</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="K305" s="24" t="n">
-        <x:v>30</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="L305" s="28"/>
       <x:c r="M305" s="29"/>
@@ -11458,7 +11456,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E306" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F306" s="21" t="str">
         <x:v>2026-06-18</x:v>
@@ -11469,10 +11467,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J306" s="24" t="n">
-        <x:v>136</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="K306" s="24" t="n">
-        <x:v>136</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="L306" s="28"/>
       <x:c r="M306" s="29"/>
@@ -11491,7 +11489,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E307" s="12" t="str">
-        <x:v>高二</x:v>
+        <x:v>高三</x:v>
       </x:c>
       <x:c r="F307" s="21" t="str">
         <x:v>2026-06-18</x:v>
@@ -11502,10 +11500,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J307" s="24" t="n">
-        <x:v>292</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="K307" s="24" t="n">
-        <x:v>292</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="L307" s="28"/>
       <x:c r="M307" s="29"/>
@@ -11521,10 +11519,10 @@
         <x:v>常规外呼</x:v>
       </x:c>
       <x:c r="D308" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>28.8</x:v>
       </x:c>
       <x:c r="E308" s="12" t="str">
-        <x:v>高三</x:v>
+        <x:v>高一</x:v>
       </x:c>
       <x:c r="F308" s="21" t="str">
         <x:v>2026-06-18</x:v>
@@ -11535,10 +11533,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J308" s="24" t="n">
-        <x:v>167</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="K308" s="24" t="n">
-        <x:v>167</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="L308" s="28"/>
       <x:c r="M308" s="29"/>
@@ -11557,7 +11555,7 @@
         <x:v>28.8</x:v>
       </x:c>
       <x:c r="E309" s="12" t="str">
-        <x:v>高一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="F309" s="21" t="str">
         <x:v>2026-06-18</x:v>
@@ -11568,79 +11566,46 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J309" s="24" t="n">
-        <x:v>92</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="K309" s="24" t="n">
-        <x:v>92</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="L309" s="28"/>
       <x:c r="M309" s="29"/>
     </x:row>
     <x:row r="310" ht="15" hidden="0" customHeight="1">
-      <x:c r="A310" s="11" t="str">
+      <x:c r="A310" s="14" t="str">
         <x:v>高中</x:v>
       </x:c>
-      <x:c r="B310" s="12" t="str">
+      <x:c r="B310" s="15" t="str">
         <x:v>暑_9</x:v>
       </x:c>
-      <x:c r="C310" s="12" t="str">
+      <x:c r="C310" s="15" t="str">
         <x:v>常规外呼</x:v>
       </x:c>
-      <x:c r="D310" s="18" t="n">
+      <x:c r="D310" s="19" t="n">
         <x:v>28.8</x:v>
       </x:c>
-      <x:c r="E310" s="12" t="str">
-        <x:v>高二</x:v>
-      </x:c>
-      <x:c r="F310" s="21" t="str">
+      <x:c r="E310" s="15" t="str">
+        <x:v>高三</x:v>
+      </x:c>
+      <x:c r="F310" s="22" t="str">
         <x:v>2026-06-18</x:v>
       </x:c>
-      <x:c r="G310" s="21"/>
-      <x:c r="H310" s="21"/>
-      <x:c r="I310" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J310" s="24" t="n">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="K310" s="24" t="n">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="L310" s="28"/>
-      <x:c r="M310" s="29"/>
-    </x:row>
-    <x:row r="311" ht="15" hidden="0" customHeight="1">
-      <x:c r="A311" s="14" t="str">
-        <x:v>高中</x:v>
-      </x:c>
-      <x:c r="B311" s="15" t="str">
-        <x:v>暑_9</x:v>
-      </x:c>
-      <x:c r="C311" s="15" t="str">
-        <x:v>常规外呼</x:v>
-      </x:c>
-      <x:c r="D311" s="19" t="n">
-        <x:v>28.8</x:v>
-      </x:c>
-      <x:c r="E311" s="15" t="str">
-        <x:v>高三</x:v>
-      </x:c>
-      <x:c r="F311" s="22" t="str">
-        <x:v>2026-06-18</x:v>
-      </x:c>
-      <x:c r="G311" s="22"/>
-      <x:c r="H311" s="22"/>
-      <x:c r="I311" s="25" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J311" s="25" t="n">
+      <x:c r="G310" s="22"/>
+      <x:c r="H310" s="22"/>
+      <x:c r="I310" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J310" s="25" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="K311" s="25" t="n">
+      <x:c r="K310" s="25" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="L311" s="30"/>
-      <x:c r="M311" s="31"/>
+      <x:c r="L310" s="30"/>
+      <x:c r="M310" s="31"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -11696,7 +11661,7 @@
         <x:v>聚合组合数</x:v>
       </x:c>
       <x:c r="B5" s="13" t="n">
-        <x:v>309</x:v>
+        <x:v>308</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -11712,7 +11677,7 @@
         <x:v>现状合计</x:v>
       </x:c>
       <x:c r="B7" s="13" t="n">
-        <x:v>85277</x:v>
+        <x:v>82884</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -11720,7 +11685,7 @@
         <x:v>完成率整体</x:v>
       </x:c>
       <x:c r="B8" s="13" t="n">
-        <x:v>1.4934676007005254</x:v>
+        <x:v>1.4515586690017512</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -11760,7 +11725,7 @@
         <x:v>最新期次现状合计</x:v>
       </x:c>
       <x:c r="B13" s="13" t="n">
-        <x:v>27157</x:v>
+        <x:v>26629</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -11768,7 +11733,7 @@
         <x:v>最新期次完成率整体</x:v>
       </x:c>
       <x:c r="B14" s="13" t="n">
-        <x:v>0.9709331426528424</x:v>
+        <x:v>0.9520557740436182</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -11888,7 +11853,7 @@
         <x:v>现状计算</x:v>
       </x:c>
       <x:c r="B29" s="13" t="str">
-        <x:v>同一统计维度下按 custom_uid 去重计数；custom_uid 缺失的行分别计数</x:v>
+        <x:v>同学部、同一期次有 target 进量日期时，仅统计下单日期不早于进量日期的 demo；同一统计维度下按 custom_uid 去重计数，custom_uid 缺失的行分别计数</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
@@ -11929,7 +11894,7 @@
         <x:v>12580</x:v>
       </x:c>
       <x:c r="C35" s="10" t="n">
-        <x:v>12189</x:v>
+        <x:v>12006</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
@@ -11940,7 +11905,7 @@
         <x:v>9450</x:v>
       </x:c>
       <x:c r="C36" s="13" t="n">
-        <x:v>9956</x:v>
+        <x:v>9611</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
@@ -11984,7 +11949,7 @@
         <x:v>12580</x:v>
       </x:c>
       <x:c r="C42" s="10" t="n">
-        <x:v>12189</x:v>
+        <x:v>12006</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
@@ -11995,7 +11960,7 @@
         <x:v>9450</x:v>
       </x:c>
       <x:c r="C43" s="13" t="n">
-        <x:v>9956</x:v>
+        <x:v>9611</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
@@ -12039,7 +12004,7 @@
         <x:v>12620</x:v>
       </x:c>
       <x:c r="C49" s="10" t="n">
-        <x:v>12641</x:v>
+        <x:v>12501</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
@@ -12050,7 +12015,7 @@
         <x:v>8665</x:v>
       </x:c>
       <x:c r="C50" s="13" t="n">
-        <x:v>7431</x:v>
+        <x:v>7306</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
@@ -12061,7 +12026,7 @@
         <x:v>4100</x:v>
       </x:c>
       <x:c r="C51" s="13" t="n">
-        <x:v>4396</x:v>
+        <x:v>4174</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
@@ -12072,7 +12037,7 @@
         <x:v>1505</x:v>
       </x:c>
       <x:c r="C52" s="13" t="n">
-        <x:v>1681</x:v>
+        <x:v>1642</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
@@ -12083,7 +12048,7 @@
         <x:v>1080</x:v>
       </x:c>
       <x:c r="C53" s="16" t="n">
-        <x:v>1008</x:v>
+        <x:v>1006</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="16.799999237060547" hidden="0" customHeight="1">
@@ -12127,7 +12092,7 @@
         <x:v>7870</x:v>
       </x:c>
       <x:c r="C59" s="13" t="n">
-        <x:v>8328</x:v>
+        <x:v>7802</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
@@ -12149,7 +12114,7 @@
         <x:v>1080</x:v>
       </x:c>
       <x:c r="C61" s="16" t="n">
-        <x:v>1008</x:v>
+        <x:v>1006</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="16.799999237060547" hidden="0" customHeight="1">
@@ -12182,7 +12147,7 @@
         <x:v>3720</x:v>
       </x:c>
       <x:c r="C66" s="10" t="n">
-        <x:v>3936</x:v>
+        <x:v>3921</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="15" hidden="0" customHeight="1">
@@ -12193,7 +12158,7 @@
         <x:v>3730</x:v>
       </x:c>
       <x:c r="C67" s="13" t="n">
-        <x:v>3580</x:v>
+        <x:v>3566</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="15" hidden="0" customHeight="1">
@@ -12204,7 +12169,7 @@
         <x:v>3510</x:v>
       </x:c>
       <x:c r="C68" s="13" t="n">
-        <x:v>3350</x:v>
+        <x:v>3342</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="15" hidden="0" customHeight="1">
@@ -12215,7 +12180,7 @@
         <x:v>2920</x:v>
       </x:c>
       <x:c r="C69" s="13" t="n">
-        <x:v>2983</x:v>
+        <x:v>2982</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="15" hidden="0" customHeight="1">
@@ -12226,7 +12191,7 @@
         <x:v>3220</x:v>
       </x:c>
       <x:c r="C70" s="13" t="n">
-        <x:v>2903</x:v>
+        <x:v>2892</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="15" hidden="0" customHeight="1">
@@ -12237,29 +12202,29 @@
         <x:v>2830</x:v>
       </x:c>
       <x:c r="C71" s="13" t="n">
-        <x:v>2790</x:v>
+        <x:v>2627</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="15" hidden="0" customHeight="1">
       <x:c r="A72" s="11" t="str">
-        <x:v>初一</x:v>
+        <x:v>高二</x:v>
       </x:c>
       <x:c r="B72" s="12" t="n">
-        <x:v>2000</x:v>
+        <x:v>2370</x:v>
       </x:c>
       <x:c r="C72" s="13" t="n">
-        <x:v>2440</x:v>
+        <x:v>2172</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="15" hidden="0" customHeight="1">
       <x:c r="A73" s="11" t="str">
-        <x:v>高二</x:v>
+        <x:v>初一</x:v>
       </x:c>
       <x:c r="B73" s="12" t="n">
-        <x:v>2370</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="C73" s="13" t="n">
-        <x:v>2172</x:v>
+        <x:v>2124</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="15" hidden="0" customHeight="1">
@@ -12416,7 +12381,7 @@
         <x:v>同一统计维度下 target 表的最晚进量日期</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A10" s="37" t="str">
         <x:v>现状</x:v>
       </x:c>
@@ -12424,7 +12389,7 @@
         <x:v>现状</x:v>
       </x:c>
       <x:c r="C10" s="39" t="str">
-        <x:v>同一统计维度下按 custom_uid 去重计数；custom_uid 缺失的行分别计数</x:v>
+        <x:v>同学部、同一期次有 target 进量日期时，仅统计下单日期不早于进量日期的 demo；同一统计维度下按 custom_uid 去重计数，custom_uid 缺失的行分别计数</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Align lec1 report with summary totals
</commit_message>
<xml_diff>
--- a/outputs/tongji_summary/tongji_summary_current.xlsx
+++ b/outputs/tongji_summary/tongji_summary_current.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目标现状对比" sheetId="1" r:id="R588ee566bb7d423e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据概览" sheetId="2" r:id="R1bba5b7693c4429e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="计算规则" sheetId="3" r:id="R009fe6ab59864e49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目标现状对比" sheetId="1" r:id="Rfcb7d7ab10034452"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据概览" sheetId="2" r:id="Rd0c4a5415cdd47b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="计算规则" sheetId="3" r:id="R6eab0f50afc34de0"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>